<commit_message>
Add bilingual disclaimer (DE/EN) to litigation cost calculator
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/publications/Litigation_Cost_Calculator_Commercial_Courts_based_on_empirical_findings.xlsx
+++ b/publications/Litigation_Cost_Calculator_Commercial_Courts_based_on_empirical_findings.xlsx
@@ -19,13 +19,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="0.000"/>
-    <numFmt numFmtId="166" formatCode="&quot;CHF &quot;#,##0"/>
-    <numFmt numFmtId="167" formatCode="0.0000"/>
-    <numFmt numFmtId="168" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="164" formatCode="&quot;CHF &quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="0.000"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -118,8 +118,19 @@
       <color rgb="00664D03"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -180,8 +191,14 @@
         <bgColor rgb="00FFF3CD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CC0000"/>
+        <bgColor rgb="00CC0000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -245,11 +262,80 @@
         <color rgb="00C9A825"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9A825"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9A825"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9A825"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9A825"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9A825"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C9A825"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C9A825"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C9A825"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9A825"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00C9A825"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -271,7 +357,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="11" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="11" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -280,14 +366,14 @@
     <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -295,10 +381,10 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="14" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="14" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="10" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -308,7 +394,7 @@
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="12" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="12" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -316,23 +402,59 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="12" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -699,7 +821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:C48"/>
+  <dimension ref="A1:C60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -707,552 +829,625 @@
     <col width="36" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="8" customHeight="1"/>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="1" t="inlineStr">
+    <row r="1" ht="8" customHeight="1">
+      <c r="A1" s="41" t="inlineStr">
+        <is>
+          <t>HAFTUNGSAUSSCHLUSS</t>
+        </is>
+      </c>
+      <c r="B1" s="42" t="n"/>
+      <c r="C1" s="42" t="n"/>
+    </row>
+    <row r="2" ht="90" customHeight="1">
+      <c r="A2" s="43" t="inlineStr">
+        <is>
+          <t>Dieses Tool dient ausschliesslich zu Informations- und Bildungszwecken. Die Kostenschätzungen basieren auf statistischen Regressionsmodellen und empirischen Daten gemäss der Studie «From Tariff to Award». Die Ergebnisse sind Näherungswerte und können erheblich von den tatsächlich zugesprochenen Prozesskosten abweichen.
+Der Autor übernimmt keinerlei Haftung für die Richtigkeit, Vollständigkeit, Aktualität oder Zuverlässigkeit der mit diesem Tool generierten Schätzungen. Die Nutzung dieses Tools stellt keine Rechtsberatung dar. Es werden keinerlei Gewährleistungen abgegeben. Für fallspezifische Kosteneinschätzungen ist eine unabhängige fachkundige Beratung einzuholen.</t>
+        </is>
+      </c>
+      <c r="B2" s="42" t="n"/>
+      <c r="C2" s="42" t="n"/>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="42" t="n"/>
+      <c r="B3" s="42" t="n"/>
+      <c r="C3" s="42" t="n"/>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="42" t="n"/>
+      <c r="B4" s="42" t="n"/>
+      <c r="C4" s="42" t="n"/>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" s="42" t="n"/>
+      <c r="B5" s="42" t="n"/>
+      <c r="C5" s="42" t="n"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="42" t="n"/>
+      <c r="B6" s="42" t="n"/>
+      <c r="C6" s="42" t="n"/>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="41" t="inlineStr">
+        <is>
+          <t>DISCLAIMER</t>
+        </is>
+      </c>
+      <c r="B7" s="42" t="n"/>
+      <c r="C7" s="42" t="n"/>
+    </row>
+    <row r="8" ht="90" customHeight="1">
+      <c r="A8" s="43" t="inlineStr">
+        <is>
+          <t>This tool is provided for informational and educational purposes only. The cost estimates are based on statistical regression models and empirical data from the study «From Tariff to Award». The results are approximations and may differ significantly from actual litigation costs awarded by the court.
+The author assumes no liability for the accuracy, completeness, timeliness, or reliability of the estimates generated by this tool. Use of this tool does not constitute legal advice. No warranties of any kind are given. For case-specific cost assessments, independent professional advice should be sought.</t>
+        </is>
+      </c>
+      <c r="B8" s="42" t="n"/>
+      <c r="C8" s="42" t="n"/>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="42" t="n"/>
+      <c r="B9" s="42" t="n"/>
+      <c r="C9" s="42" t="n"/>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="42" t="n"/>
+      <c r="B10" s="42" t="n"/>
+      <c r="C10" s="42" t="n"/>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="42" t="n"/>
+      <c r="B11" s="42" t="n"/>
+      <c r="C11" s="42" t="n"/>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="42" t="n"/>
+      <c r="B12" s="42" t="n"/>
+      <c r="C12" s="42" t="n"/>
+    </row>
+    <row r="13" ht="24" customHeight="1"/>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>Prozesskostenrechner</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Ordentliche Verfahren vor den Handelsgerichten Zürich und Aargau — Modell 6</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Bitte füllen Sie die gelb markierten Felder aus. Die Ergebnisse werden automatisch berechnet. Das Tool schätzt Gerichtskosten (vom Gericht festgesetzt) und Parteientschädigung (Anwaltskostenersatz an die obsiegende Partei) auf Basis von über 900 Urteilen.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="26" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">   EINGABE</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Fall</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="7" t="n"/>
-    </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
-        <is>
-          <t>Kanton</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>Zürich</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>Standort des zuständigen Handelsgerichts</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>Streitwert (CHF)</t>
-        </is>
-      </c>
-      <c r="B8" s="11" t="n">
-        <v>500000</v>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>Gesamtwert aller Rechtsbegehren</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t>Rechtsgebiet</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Forderung Dienstleistungen</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>Hauptkategorie gemäss Urteilskopf</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>Kläger mit Sitz in der Schweiz</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>Sitz oder Wohnsitz in der Schweiz?</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>Beklagter mit Sitz in der Schweiz</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>Sitz oder Wohnsitz in der Schweiz?</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>Anzahl Kläger</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>inkl. allfälliger Streitgenossen</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>Anzahl Beklagte</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>inkl. allfälliger Streitgenossen</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Verfahrensgang (erwartete oder eingetretene Prozessschritte)</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="n"/>
-      <c r="C14" s="7" t="n"/>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Klagantwort eingereicht</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="C15" s="10" t="inlineStr">
-        <is>
-          <t>Hat der Beklagte eine Klagantwort eingereicht?</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>Zweiter Schriftenwechsel</t>
-        </is>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Nein</t>
-        </is>
-      </c>
-      <c r="C16" s="10" t="inlineStr">
-        <is>
-          <t>Replik und Duplik angeordnet?</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="8" t="inlineStr">
-        <is>
-          <t>Widerklage erhoben</t>
-        </is>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Nein</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>Hat der Beklagte eine Widerklage erhoben?</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>Widerklage mit 2. Schriftenwechsel</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Nein</t>
-        </is>
-      </c>
-      <c r="C18" s="10" t="inlineStr">
-        <is>
-          <t>Zweiter Schriftenwechsel zur Widerklage?</t>
-        </is>
-      </c>
+      <c r="B18" s="7" t="n"/>
+      <c r="C18" s="7" t="n"/>
     </row>
     <row r="19" ht="24" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Zusätzliche Eingaben</t>
+          <t>Kanton</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>Nein</t>
+          <t>Zürich</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Weitere Eingaben über die Schriftenw. hinaus?</t>
+          <t>Standort des zuständigen Handelsgerichts</t>
         </is>
       </c>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Vergleichsverhandlung</t>
-        </is>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>Nein</t>
-        </is>
+          <t>Streitwert (CHF)</t>
+        </is>
+      </c>
+      <c r="B20" s="44" t="n">
+        <v>500000</v>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Wurde eine Vergleichsverhandlung durchgeführt?</t>
+          <t>Gesamtwert aller Rechtsbegehren</t>
         </is>
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Gutachten</t>
+          <t>Rechtsgebiet</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Nein</t>
+          <t>Forderung Dienstleistungen</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Wurde ein Sachverständigengutachten eingeholt?</t>
+          <t>Hauptkategorie gemäss Urteilskopf</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Kostenverteilung</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="n"/>
-      <c r="C22" s="7" t="n"/>
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Kläger mit Sitz in der Schweiz</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>Sitz oder Wohnsitz in der Schweiz?</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
+          <t>Beklagter mit Sitz in der Schweiz</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>Sitz oder Wohnsitz in der Schweiz?</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="10" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Anzahl Kläger</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>inkl. allfälliger Streitgenossen</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="26" customHeight="1">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Anzahl Beklagte</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>inkl. allfälliger Streitgenossen</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Verfahrensgang (erwartete oder eingetretene Prozessschritte)</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n"/>
+      <c r="C26" s="7" t="n"/>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>Klagantwort eingereicht</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Hat der Beklagte eine Klagantwort eingereicht?</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="6" customHeight="1">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>Zweiter Schriftenwechsel</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>Replik und Duplik angeordnet?</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>Widerklage erhoben</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>Hat der Beklagte eine Widerklage erhoben?</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Widerklage mit 2. Schriftenwechsel</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>Zweiter Schriftenwechsel zur Widerklage?</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="4" customHeight="1">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>Zusätzliche Eingaben</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="C31" s="10" t="inlineStr">
+        <is>
+          <t>Weitere Eingaben über die Schriftenw. hinaus?</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>Vergleichsverhandlung</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>Wurde eine Vergleichsverhandlung durchgeführt?</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Gutachten</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>Wurde ein Sachverständigengutachten eingeholt?</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Kostenverteilung</t>
+        </is>
+      </c>
+      <c r="B34" s="7" t="n"/>
+      <c r="C34" s="7" t="n"/>
+    </row>
+    <row r="35" ht="26" customHeight="1">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
           <t>Unterliegensquote Kläger (0–1)</t>
         </is>
       </c>
-      <c r="B23" s="12" t="n">
+      <c r="B35" s="12" t="n">
         <v>0.5</v>
       </c>
-      <c r="C23" s="10" t="inlineStr">
+      <c r="C35" s="10" t="inlineStr">
         <is>
           <t>0 = Kl. obsiegt, 1 = Kl. unterliegt (beeinflusst nur PE)</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="10" customHeight="1"/>
-    <row r="25" ht="26" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="36" ht="6" customHeight="1"/>
+    <row r="37" ht="24" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">   ERGEBNISSE</t>
         </is>
       </c>
-      <c r="B25" s="5" t="n"/>
-      <c r="C25" s="5" t="n"/>
-    </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="13" t="inlineStr">
+    </row>
+    <row r="38" ht="24" customHeight="1">
+      <c r="A38" s="13" t="inlineStr">
         <is>
           <t>Gerichtskosten gemäss Tarif</t>
         </is>
       </c>
-      <c r="B26" s="14">
+      <c r="B38" s="45">
         <f>IF(B7="Zürich",MAX(150,INDEX(Tarif!C$3:C$10,MATCH(B8,Tarif!A$3:A$10,1))+(B8-INDEX(Tarif!A$3:A$10,MATCH(B8,Tarif!A$3:A$10,1)))*INDEX(Tarif!D$3:D$10,MATCH(B8,Tarif!A$3:A$10,1))),INDEX(Tarif!C$19:C$28,MATCH(B8,Tarif!A$19:A$28,1))+B8*INDEX(Tarif!D$19:D$28,MATCH(B8,Tarif!A$19:A$28,1)))</f>
         <v/>
       </c>
-      <c r="C26" s="15" t="inlineStr">
+      <c r="C38" s="15" t="inlineStr">
         <is>
           <t>Gesetzlicher Ausgangswert (GebV OG ZH / GebT AG)</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="13" t="inlineStr">
+    <row r="39" ht="10" customHeight="1">
+      <c r="A39" s="13" t="inlineStr">
         <is>
           <t>Parteientschädigung gemäss Tarif</t>
         </is>
       </c>
-      <c r="B27" s="14">
+      <c r="B39" s="45">
         <f>IF(B7="Zürich",MAX(100,INDEX(Tarif!H$3:H$14,MATCH(B8,Tarif!F$3:F$14,1))+(B8-INDEX(Tarif!F$3:F$14,MATCH(B8,Tarif!F$3:F$14,1)))*INDEX(Tarif!I$3:I$14,MATCH(B8,Tarif!F$3:F$14,1))),INDEX(Tarif!H$19:H$30,MATCH(B8,Tarif!F$19:F$30,1))+B8*INDEX(Tarif!I$19:I$30,MATCH(B8,Tarif!F$19:F$30,1)))</f>
         <v/>
       </c>
-      <c r="C27" s="15" t="inlineStr">
+      <c r="C39" s="15" t="inlineStr">
         <is>
           <t>Gesetzlicher Ausgangswert (AnwGebV ZH / AnwT AG)</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="6" customHeight="1"/>
-    <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="13" t="inlineStr">
+    <row r="40" ht="18" customHeight="1"/>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="13" t="inlineStr">
         <is>
           <t>Geschätzte Gerichtskosten</t>
         </is>
       </c>
-      <c r="B29" s="14">
+      <c r="B41" s="45">
         <f>B26*EXP(B47)</f>
         <v/>
       </c>
-      <c r="C29" s="15" t="inlineStr">
+      <c r="C41" s="15" t="inlineStr">
         <is>
           <t>Modellschätzung basierend auf 976 Urteilen</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="24" customHeight="1">
-      <c r="A30" s="13" t="inlineStr">
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="13" t="inlineStr">
         <is>
           <t>Geschätzte Parteientschädigung</t>
         </is>
       </c>
-      <c r="B30" s="14">
+      <c r="B42" s="45">
         <f>B27*EXP(B48)</f>
         <v/>
       </c>
-      <c r="C30" s="15" t="inlineStr">
+      <c r="C42" s="15" t="inlineStr">
         <is>
           <t>Modellschätzung basierend auf 898 Urteilen</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="4" customHeight="1"/>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="16" t="inlineStr">
+    <row r="43" ht="18" customHeight="1"/>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="16" t="inlineStr">
         <is>
           <t>GESCHÄTZTE GESAMTKOSTEN</t>
         </is>
       </c>
-      <c r="B32" s="17">
+      <c r="B44" s="46">
         <f>B29+B30</f>
         <v/>
       </c>
-      <c r="C32" s="18" t="inlineStr">
+      <c r="C44" s="18" t="inlineStr">
         <is>
           <t>Summe GK + PE (ohne eigene Anwaltskosten)</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="19" t="inlineStr">
+    <row r="45" ht="16" customHeight="1">
+      <c r="A45" s="19" t="inlineStr">
         <is>
           <t>Bandbreite: In 50% der Fälle liegen die tatsächlichen Kosten innerhalb dieses Bereichs.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="26" customHeight="1">
-      <c r="A34" s="20" t="inlineStr">
+    <row r="46" ht="16" customHeight="1">
+      <c r="A46" s="20" t="inlineStr">
         <is>
           <t>Bandbreite Gerichtskosten (±21%)</t>
         </is>
       </c>
-      <c r="B34" s="21">
+      <c r="B46" s="47">
         <f>B29*(1-0.21)</f>
         <v/>
       </c>
-      <c r="C34" s="21">
+      <c r="C46" s="47">
         <f>B29*(1+0.21)</f>
         <v/>
       </c>
     </row>
-    <row r="35" ht="26" customHeight="1">
-      <c r="A35" s="20" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="20" t="inlineStr">
         <is>
           <t>Bandbreite Parteientschädigung (±25.8%)</t>
         </is>
       </c>
-      <c r="B35" s="21">
+      <c r="B47" s="47">
         <f>B30*(1-0.258)</f>
         <v/>
       </c>
-      <c r="C35" s="21">
+      <c r="C47" s="47">
         <f>B30*(1+0.258)</f>
         <v/>
       </c>
     </row>
-    <row r="36" ht="6" customHeight="1"/>
-    <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="13" t="inlineStr">
+    <row r="48"/>
+    <row r="49">
+      <c r="A49" s="13" t="inlineStr">
         <is>
           <t>Abweichung vom Tarif — Gerichtskosten</t>
         </is>
       </c>
-      <c r="B37" s="22">
+      <c r="B49" s="48">
         <f>(B29-B26)/B26</f>
         <v/>
       </c>
-      <c r="C37" s="15" t="inlineStr">
+      <c r="C49" s="15" t="inlineStr">
         <is>
           <t>positiv = über Tarif, negativ = unter Tarif</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="24" customHeight="1">
-      <c r="A38" s="13" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="13" t="inlineStr">
         <is>
           <t>Abweichung vom Tarif — Parteientschädigung</t>
         </is>
       </c>
-      <c r="B38" s="22">
+      <c r="B50" s="48">
         <f>(B30-B27)/B27</f>
         <v/>
       </c>
-      <c r="C38" s="15" t="inlineStr">
+      <c r="C50" s="15" t="inlineStr">
         <is>
           <t>positiv = über Tarif, negativ = unter Tarif</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="10" customHeight="1"/>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="23" t="inlineStr">
+    <row r="51"/>
+    <row r="52">
+      <c r="A52" s="23" t="inlineStr">
         <is>
           <t>HAFTUNGSAUSSCHLUSS: Dieses Tool dient ausschliesslich zu Informations- und Bildungszwecken. Die Kostenschätzungen basieren auf statistischen Regressionsmodellen und empirischen Daten gemäss der Studie «From Tariff to Award». Die Ergebnisse sind Näherungswerte und können erheblich von den tatsächlich zugesprochenen Prozesskosten abweichen.
 Der Autor übernimmt keinerlei Haftung für die Richtigkeit, Vollständigkeit, Aktualität oder Zuverlässigkeit der mit diesem Tool generierten Schätzungen. Die Nutzung dieses Tools stellt keine Rechtsberatung dar. Es werden keinerlei Gewährleistungen abgegeben. Für fallspezifische Kosteneinschätzungen ist eine unabhängige fachkundige Beratung einzuholen.</t>
         </is>
       </c>
-      <c r="B40" s="24" t="n"/>
-      <c r="C40" s="24" t="n"/>
-    </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="24" t="n"/>
-      <c r="B41" s="24" t="n"/>
-      <c r="C41" s="24" t="n"/>
-    </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="24" t="n"/>
-      <c r="B42" s="24" t="n"/>
-      <c r="C42" s="24" t="n"/>
-    </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="24" t="n"/>
-      <c r="B43" s="24" t="n"/>
-      <c r="C43" s="24" t="n"/>
-    </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="24" t="n"/>
-      <c r="B44" s="24" t="n"/>
-      <c r="C44" s="24" t="n"/>
-    </row>
-    <row r="45" ht="16" customHeight="1">
-      <c r="A45" s="19" t="inlineStr">
+      <c r="B52" s="49" t="n"/>
+      <c r="C52" s="50" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="51" t="n"/>
+      <c r="C53" s="52" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="51" t="n"/>
+      <c r="C54" s="52" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="51" t="n"/>
+      <c r="C55" s="52" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="53" t="n"/>
+      <c r="B56" s="54" t="n"/>
+      <c r="C56" s="55" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="19" t="inlineStr">
         <is>
           <t>Grundlage: «From Tariff to Award» — Modell 6 (Year FE + Judge FE). Medianer abs. Prognosefehler: GK 21%, PE 25.8%.</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="16" customHeight="1">
-      <c r="A46" s="25" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="25" t="inlineStr">
         <is>
           <t>HILFSBERECHNUNGEN</t>
         </is>
       </c>
-      <c r="B46" s="26" t="n"/>
-      <c r="C46" s="26" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="27" t="inlineStr">
+      <c r="B58" s="26" t="n"/>
+      <c r="C58" s="26" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="27" t="inlineStr">
         <is>
           <t>ln(GK / Grundtarif)</t>
         </is>
       </c>
-      <c r="B47" s="28">
+      <c r="B59" s="56">
         <f>Koeffizienten!B3+LN(B26)*Koeffizienten!B4+IF(B7="Aargau",1,0)*Koeffizienten!B5+IF(B7="Aargau",1,0)*LN(B26)*Koeffizienten!B6+INDEX(Koeffizienten!B$31:B$39,MATCH(B9,Koeffizienten!A$31:A$39,0))+IF(B10="Ja",1,0)*Koeffizienten!B9+IF(B11="Ja",1,0)*Koeffizienten!B10+LN(MAX(1,B12))*Koeffizienten!B7+LN(MAX(1,B13))*Koeffizienten!B8+IF(B15="Ja",1,0)*Koeffizienten!B19+IF(B16="Ja",1,0)*Koeffizienten!B20+IF(B17="Ja",1,0)*Koeffizienten!B21+IF(B18="Ja",1,0)*Koeffizienten!B22+IF(B19="Ja",1,0)*Koeffizienten!B23+IF(B20="Ja",1,0)*Koeffizienten!B24+IF(B21="Ja",1,0)*Koeffizienten!B25</f>
         <v/>
       </c>
-      <c r="C47" s="26" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="27" t="inlineStr">
+      <c r="C59" s="26" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="27" t="inlineStr">
         <is>
           <t>ln(PE / Grundtarif)</t>
         </is>
       </c>
-      <c r="B48" s="28">
+      <c r="B60" s="56">
         <f>Koeffizienten!C3+LN(B27)*Koeffizienten!C4+IF(B7="Aargau",1,0)*Koeffizienten!C5+IF(B7="Aargau",1,0)*LN(B27)*Koeffizienten!C6+INDEX(Koeffizienten!C$31:C$39,MATCH(B9,Koeffizienten!A$31:A$39,0))+IF(B10="Ja",1,0)*Koeffizienten!C9+IF(B11="Ja",1,0)*Koeffizienten!C10+LN(MAX(1,B12))*Koeffizienten!C7+LN(MAX(1,B13))*Koeffizienten!C8+IF(B15="Ja",1,0)*Koeffizienten!C19+IF(B16="Ja",1,0)*Koeffizienten!C20+IF(B17="Ja",1,0)*Koeffizienten!C21+IF(B18="Ja",1,0)*Koeffizienten!C22+IF(B19="Ja",1,0)*Koeffizienten!C23+IF(B20="Ja",1,0)*Koeffizienten!C24+IF(B21="Ja",1,0)*Koeffizienten!C25+B23*Koeffizienten!C26</f>
         <v/>
       </c>
-      <c r="C48" s="26" t="n"/>
+      <c r="C60" s="26" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="10">
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="A33:C33"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="A40:C44"/>
+    <mergeCell ref="A2:C6"/>
     <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A8:C12"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
@@ -1308,17 +1503,11 @@
           <t>ZH Gerichtskosten (GebV OG ZH)</t>
         </is>
       </c>
-      <c r="B1" s="5" t="n"/>
-      <c r="C1" s="5" t="n"/>
-      <c r="D1" s="5" t="n"/>
       <c r="F1" s="29" t="inlineStr">
         <is>
           <t>ZH Parteientschädigung (AnwGebV ZH)</t>
         </is>
       </c>
-      <c r="G1" s="5" t="n"/>
-      <c r="H1" s="5" t="n"/>
-      <c r="I1" s="5" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="30" t="inlineStr">
@@ -1372,7 +1561,7 @@
       <c r="C3" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="D3" s="32" t="n">
+      <c r="D3" s="57" t="n">
         <v>0.25</v>
       </c>
       <c r="F3" s="31" t="n">
@@ -1384,7 +1573,7 @@
       <c r="H3" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="I3" s="32" t="n">
+      <c r="I3" s="57" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -1398,7 +1587,7 @@
       <c r="C4" s="33" t="n">
         <v>250</v>
       </c>
-      <c r="D4" s="34" t="n">
+      <c r="D4" s="58" t="n">
         <v>0.2</v>
       </c>
       <c r="F4" s="33" t="n">
@@ -1410,7 +1599,7 @@
       <c r="H4" s="33" t="n">
         <v>1250</v>
       </c>
-      <c r="I4" s="34" t="n">
+      <c r="I4" s="58" t="n">
         <v>0.23</v>
       </c>
     </row>
@@ -1424,7 +1613,7 @@
       <c r="C5" s="31" t="n">
         <v>1050</v>
       </c>
-      <c r="D5" s="32" t="n">
+      <c r="D5" s="57" t="n">
         <v>0.14</v>
       </c>
       <c r="F5" s="31" t="n">
@@ -1436,7 +1625,7 @@
       <c r="H5" s="31" t="n">
         <v>2400</v>
       </c>
-      <c r="I5" s="32" t="n">
+      <c r="I5" s="57" t="n">
         <v>0.15</v>
       </c>
     </row>
@@ -1450,7 +1639,7 @@
       <c r="C6" s="33" t="n">
         <v>3150</v>
       </c>
-      <c r="D6" s="34" t="n">
+      <c r="D6" s="58" t="n">
         <v>0.08</v>
       </c>
       <c r="F6" s="33" t="n">
@@ -1462,7 +1651,7 @@
       <c r="H6" s="33" t="n">
         <v>3900</v>
       </c>
-      <c r="I6" s="34" t="n">
+      <c r="I6" s="58" t="n">
         <v>0.11</v>
       </c>
     </row>
@@ -1476,7 +1665,7 @@
       <c r="C7" s="31" t="n">
         <v>7950</v>
       </c>
-      <c r="D7" s="32" t="n">
+      <c r="D7" s="57" t="n">
         <v>0.04</v>
       </c>
       <c r="F7" s="31" t="n">
@@ -1488,7 +1677,7 @@
       <c r="H7" s="31" t="n">
         <v>6100</v>
       </c>
-      <c r="I7" s="32" t="n">
+      <c r="I7" s="57" t="n">
         <v>0.09</v>
       </c>
     </row>
@@ -1502,7 +1691,7 @@
       <c r="C8" s="33" t="n">
         <v>16750</v>
       </c>
-      <c r="D8" s="34" t="n">
+      <c r="D8" s="58" t="n">
         <v>0.02</v>
       </c>
       <c r="F8" s="33" t="n">
@@ -1514,7 +1703,7 @@
       <c r="H8" s="33" t="n">
         <v>9700</v>
       </c>
-      <c r="I8" s="34" t="n">
+      <c r="I8" s="58" t="n">
         <v>0.06</v>
       </c>
     </row>
@@ -1528,7 +1717,7 @@
       <c r="C9" s="31" t="n">
         <v>30750</v>
       </c>
-      <c r="D9" s="32" t="n">
+      <c r="D9" s="57" t="n">
         <v>0.01</v>
       </c>
       <c r="F9" s="31" t="n">
@@ -1540,7 +1729,7 @@
       <c r="H9" s="31" t="n">
         <v>14500</v>
       </c>
-      <c r="I9" s="32" t="n">
+      <c r="I9" s="57" t="n">
         <v>0.035</v>
       </c>
     </row>
@@ -1554,7 +1743,7 @@
       <c r="C10" s="33" t="n">
         <v>120750</v>
       </c>
-      <c r="D10" s="34" t="n">
+      <c r="D10" s="58" t="n">
         <v>0.005</v>
       </c>
       <c r="F10" s="33" t="n">
@@ -1566,7 +1755,7 @@
       <c r="H10" s="33" t="n">
         <v>19400</v>
       </c>
-      <c r="I10" s="34" t="n">
+      <c r="I10" s="58" t="n">
         <v>0.02</v>
       </c>
     </row>
@@ -1580,7 +1769,7 @@
       <c r="H11" s="31" t="n">
         <v>25400</v>
       </c>
-      <c r="I11" s="32" t="n">
+      <c r="I11" s="57" t="n">
         <v>0.015</v>
       </c>
     </row>
@@ -1594,7 +1783,7 @@
       <c r="H12" s="33" t="n">
         <v>31400</v>
       </c>
-      <c r="I12" s="34" t="n">
+      <c r="I12" s="58" t="n">
         <v>0.01</v>
       </c>
     </row>
@@ -1608,7 +1797,7 @@
       <c r="H13" s="31" t="n">
         <v>61400</v>
       </c>
-      <c r="I13" s="32" t="n">
+      <c r="I13" s="57" t="n">
         <v>0.0075</v>
       </c>
     </row>
@@ -1622,7 +1811,7 @@
       <c r="H14" s="33" t="n">
         <v>106400</v>
       </c>
-      <c r="I14" s="34" t="n">
+      <c r="I14" s="58" t="n">
         <v>0.005</v>
       </c>
     </row>
@@ -1632,17 +1821,11 @@
           <t>AG Gerichtskosten (GebT AG)</t>
         </is>
       </c>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
       <c r="F17" s="29" t="inlineStr">
         <is>
           <t>AG Parteientschädigung (AnwT AG)</t>
         </is>
       </c>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="30" t="inlineStr">
@@ -1696,7 +1879,7 @@
       <c r="C19" s="31" t="n">
         <v>900</v>
       </c>
-      <c r="D19" s="32" t="n">
+      <c r="D19" s="57" t="n">
         <v>0.11</v>
       </c>
       <c r="F19" s="31" t="n">
@@ -1708,7 +1891,7 @@
       <c r="H19" s="31" t="n">
         <v>1110</v>
       </c>
-      <c r="I19" s="32" t="n">
+      <c r="I19" s="57" t="n">
         <v>0.22</v>
       </c>
     </row>
@@ -1722,7 +1905,7 @@
       <c r="C20" s="33" t="n">
         <v>1160</v>
       </c>
-      <c r="D20" s="34" t="n">
+      <c r="D20" s="58" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="F20" s="33" t="n">
@@ -1734,7 +1917,7 @@
       <c r="H20" s="33" t="n">
         <v>1230</v>
       </c>
-      <c r="I20" s="34" t="n">
+      <c r="I20" s="58" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1748,7 +1931,7 @@
       <c r="C21" s="31" t="n">
         <v>1290</v>
       </c>
-      <c r="D21" s="32" t="n">
+      <c r="D21" s="57" t="n">
         <v>0.06</v>
       </c>
       <c r="F21" s="31" t="n">
@@ -1760,7 +1943,7 @@
       <c r="H21" s="31" t="n">
         <v>1850</v>
       </c>
-      <c r="I21" s="32" t="n">
+      <c r="I21" s="57" t="n">
         <v>0.15</v>
       </c>
     </row>
@@ -1774,7 +1957,7 @@
       <c r="C22" s="33" t="n">
         <v>770</v>
       </c>
-      <c r="D22" s="34" t="n">
+      <c r="D22" s="58" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="F22" s="33" t="n">
@@ -1786,7 +1969,7 @@
       <c r="H22" s="33" t="n">
         <v>2590</v>
       </c>
-      <c r="I22" s="34" t="n">
+      <c r="I22" s="58" t="n">
         <v>0.12</v>
       </c>
     </row>
@@ -1800,7 +1983,7 @@
       <c r="C23" s="31" t="n">
         <v>4270</v>
       </c>
-      <c r="D23" s="32" t="n">
+      <c r="D23" s="57" t="n">
         <v>0.035</v>
       </c>
       <c r="F23" s="31" t="n">
@@ -1812,7 +1995,7 @@
       <c r="H23" s="31" t="n">
         <v>4070</v>
       </c>
-      <c r="I23" s="32" t="n">
+      <c r="I23" s="57" t="n">
         <v>0.09</v>
       </c>
     </row>
@@ -1826,7 +2009,7 @@
       <c r="C24" s="33" t="n">
         <v>6870</v>
       </c>
-      <c r="D24" s="34" t="n">
+      <c r="D24" s="58" t="n">
         <v>0.022</v>
       </c>
       <c r="F24" s="33" t="n">
@@ -1838,7 +2021,7 @@
       <c r="H24" s="33" t="n">
         <v>6530</v>
       </c>
-      <c r="I24" s="34" t="n">
+      <c r="I24" s="58" t="n">
         <v>0.064</v>
       </c>
     </row>
@@ -1852,7 +2035,7 @@
       <c r="C25" s="31" t="n">
         <v>9670</v>
       </c>
-      <c r="D25" s="32" t="n">
+      <c r="D25" s="57" t="n">
         <v>0.015</v>
       </c>
       <c r="F25" s="31" t="n">
@@ -1864,7 +2047,7 @@
       <c r="H25" s="31" t="n">
         <v>10230</v>
       </c>
-      <c r="I25" s="32" t="n">
+      <c r="I25" s="57" t="n">
         <v>0.044</v>
       </c>
     </row>
@@ -1878,7 +2061,7 @@
       <c r="C26" s="33" t="n">
         <v>13670</v>
       </c>
-      <c r="D26" s="34" t="n">
+      <c r="D26" s="58" t="n">
         <v>0.01</v>
       </c>
       <c r="F26" s="33" t="n">
@@ -1890,7 +2073,7 @@
       <c r="H26" s="33" t="n">
         <v>14300</v>
       </c>
-      <c r="I26" s="34" t="n">
+      <c r="I26" s="58" t="n">
         <v>0.033</v>
       </c>
     </row>
@@ -1904,7 +2087,7 @@
       <c r="C27" s="31" t="n">
         <v>21670</v>
       </c>
-      <c r="D27" s="32" t="n">
+      <c r="D27" s="57" t="n">
         <v>0.005</v>
       </c>
       <c r="F27" s="31" t="n">
@@ -1916,7 +2099,7 @@
       <c r="H27" s="31" t="n">
         <v>20240</v>
       </c>
-      <c r="I27" s="32" t="n">
+      <c r="I27" s="57" t="n">
         <v>0.025</v>
       </c>
     </row>
@@ -1930,7 +2113,7 @@
       <c r="C28" s="33" t="n">
         <v>28270</v>
       </c>
-      <c r="D28" s="34" t="n">
+      <c r="D28" s="58" t="n">
         <v>0.003</v>
       </c>
       <c r="F28" s="33" t="n">
@@ -1942,7 +2125,7 @@
       <c r="H28" s="33" t="n">
         <v>29040</v>
       </c>
-      <c r="I28" s="34" t="n">
+      <c r="I28" s="58" t="n">
         <v>0.019</v>
       </c>
     </row>
@@ -1956,7 +2139,7 @@
       <c r="H29" s="31" t="n">
         <v>44440</v>
       </c>
-      <c r="I29" s="32" t="n">
+      <c r="I29" s="57" t="n">
         <v>0.014</v>
       </c>
     </row>
@@ -1970,7 +2153,7 @@
       <c r="H30" s="33" t="n">
         <v>69080</v>
       </c>
-      <c r="I30" s="34" t="n">
+      <c r="I30" s="58" t="n">
         <v>0.01</v>
       </c>
     </row>
@@ -2046,10 +2229,10 @@
           <t>Intercept</t>
         </is>
       </c>
-      <c r="B3" s="37" t="n">
+      <c r="B3" s="59" t="n">
         <v>0.927</v>
       </c>
-      <c r="C3" s="37" t="n">
+      <c r="C3" s="59" t="n">
         <v>1.888</v>
       </c>
     </row>
@@ -2059,10 +2242,10 @@
           <t>ln(Baseline)</t>
         </is>
       </c>
-      <c r="B4" s="39" t="n">
+      <c r="B4" s="60" t="n">
         <v>-0.111</v>
       </c>
-      <c r="C4" s="39" t="n">
+      <c r="C4" s="60" t="n">
         <v>-0.17</v>
       </c>
     </row>
@@ -2072,10 +2255,10 @@
           <t>D_AG</t>
         </is>
       </c>
-      <c r="B5" s="37" t="n">
+      <c r="B5" s="59" t="n">
         <v>-0.518</v>
       </c>
-      <c r="C5" s="37" t="n">
+      <c r="C5" s="59" t="n">
         <v>-3.414</v>
       </c>
     </row>
@@ -2085,10 +2268,10 @@
           <t>D_AG x ln(Baseline)</t>
         </is>
       </c>
-      <c r="B6" s="39" t="n">
+      <c r="B6" s="60" t="n">
         <v>0.057</v>
       </c>
-      <c r="C6" s="39" t="n">
+      <c r="C6" s="60" t="n">
         <v>0.463</v>
       </c>
     </row>
@@ -2098,10 +2281,10 @@
           <t>ln(Kläger)</t>
         </is>
       </c>
-      <c r="B7" s="37" t="n">
+      <c r="B7" s="59" t="n">
         <v>0.052</v>
       </c>
-      <c r="C7" s="37" t="n">
+      <c r="C7" s="59" t="n">
         <v>-0.13</v>
       </c>
     </row>
@@ -2111,10 +2294,10 @@
           <t>ln(Beklagte)</t>
         </is>
       </c>
-      <c r="B8" s="39" t="n">
+      <c r="B8" s="60" t="n">
         <v>0.092</v>
       </c>
-      <c r="C8" s="39" t="n">
+      <c r="C8" s="60" t="n">
         <v>0.176</v>
       </c>
     </row>
@@ -2124,10 +2307,10 @@
           <t>Domizil Kläger</t>
         </is>
       </c>
-      <c r="B9" s="37" t="n">
+      <c r="B9" s="59" t="n">
         <v>-0.08599999999999999</v>
       </c>
-      <c r="C9" s="37" t="n">
+      <c r="C9" s="59" t="n">
         <v>-0.129</v>
       </c>
     </row>
@@ -2137,10 +2320,10 @@
           <t>Domizil Beklagter</t>
         </is>
       </c>
-      <c r="B10" s="39" t="n">
+      <c r="B10" s="60" t="n">
         <v>-0.079</v>
       </c>
-      <c r="C10" s="39" t="n">
+      <c r="C10" s="60" t="n">
         <v>-0.022</v>
       </c>
     </row>
@@ -2150,10 +2333,10 @@
           <t>D_Bau</t>
         </is>
       </c>
-      <c r="B11" s="37" t="n">
+      <c r="B11" s="59" t="n">
         <v>0.037</v>
       </c>
-      <c r="C11" s="37" t="n">
+      <c r="C11" s="59" t="n">
         <v>-0.208</v>
       </c>
     </row>
@@ -2163,10 +2346,10 @@
           <t>D_Handel</t>
         </is>
       </c>
-      <c r="B12" s="39" t="n">
+      <c r="B12" s="60" t="n">
         <v>0.007</v>
       </c>
-      <c r="C12" s="39" t="n">
+      <c r="C12" s="60" t="n">
         <v>0.004</v>
       </c>
     </row>
@@ -2176,10 +2359,10 @@
           <t>D_Finanz/Versicherung</t>
         </is>
       </c>
-      <c r="B13" s="37" t="n">
+      <c r="B13" s="59" t="n">
         <v>0.068</v>
       </c>
-      <c r="C13" s="37" t="n">
+      <c r="C13" s="59" t="n">
         <v>-0.12</v>
       </c>
     </row>
@@ -2189,10 +2372,10 @@
           <t>D_Organhaftung</t>
         </is>
       </c>
-      <c r="B14" s="39" t="n">
+      <c r="B14" s="60" t="n">
         <v>-0.006</v>
       </c>
-      <c r="C14" s="39" t="n">
+      <c r="C14" s="60" t="n">
         <v>-0.064</v>
       </c>
     </row>
@@ -2202,10 +2385,10 @@
           <t>D_UWG/URG</t>
         </is>
       </c>
-      <c r="B15" s="37" t="n">
+      <c r="B15" s="59" t="n">
         <v>0.592</v>
       </c>
-      <c r="C15" s="37" t="n">
+      <c r="C15" s="59" t="n">
         <v>1.058</v>
       </c>
     </row>
@@ -2215,10 +2398,10 @@
           <t>D_Immaterialgüterrecht</t>
         </is>
       </c>
-      <c r="B16" s="39" t="n">
+      <c r="B16" s="60" t="n">
         <v>0.06900000000000001</v>
       </c>
-      <c r="C16" s="39" t="n">
+      <c r="C16" s="60" t="n">
         <v>-0.079</v>
       </c>
     </row>
@@ -2228,10 +2411,10 @@
           <t>D_Gesellschaftsrecht</t>
         </is>
       </c>
-      <c r="B17" s="37" t="n">
+      <c r="B17" s="59" t="n">
         <v>-0.227</v>
       </c>
-      <c r="C17" s="37" t="n">
+      <c r="C17" s="59" t="n">
         <v>-0.045</v>
       </c>
     </row>
@@ -2241,10 +2424,10 @@
           <t>D_Übrige</t>
         </is>
       </c>
-      <c r="B18" s="39" t="n">
+      <c r="B18" s="60" t="n">
         <v>0.029</v>
       </c>
-      <c r="C18" s="39" t="n">
+      <c r="C18" s="60" t="n">
         <v>-0.159</v>
       </c>
     </row>
@@ -2254,10 +2437,10 @@
           <t>Klagantwort</t>
         </is>
       </c>
-      <c r="B19" s="37" t="n">
+      <c r="B19" s="59" t="n">
         <v>-0.08799999999999999</v>
       </c>
-      <c r="C19" s="37" t="n">
+      <c r="C19" s="59" t="n">
         <v>-0.004</v>
       </c>
     </row>
@@ -2267,10 +2450,10 @@
           <t>Zweiter Schriftenwechsel</t>
         </is>
       </c>
-      <c r="B20" s="39" t="n">
+      <c r="B20" s="60" t="n">
         <v>0.504</v>
       </c>
-      <c r="C20" s="39" t="n">
+      <c r="C20" s="60" t="n">
         <v>0.319</v>
       </c>
     </row>
@@ -2280,10 +2463,10 @@
           <t>Widerklage</t>
         </is>
       </c>
-      <c r="B21" s="37" t="n">
+      <c r="B21" s="59" t="n">
         <v>-0.159</v>
       </c>
-      <c r="C21" s="37" t="n">
+      <c r="C21" s="59" t="n">
         <v>-0.173</v>
       </c>
     </row>
@@ -2293,10 +2476,10 @@
           <t>Widerklage 2. SW</t>
         </is>
       </c>
-      <c r="B22" s="39" t="n">
+      <c r="B22" s="60" t="n">
         <v>0.395</v>
       </c>
-      <c r="C22" s="39" t="n">
+      <c r="C22" s="60" t="n">
         <v>0.192</v>
       </c>
     </row>
@@ -2306,10 +2489,10 @@
           <t>Zusätzliche Eingaben</t>
         </is>
       </c>
-      <c r="B23" s="37" t="n">
+      <c r="B23" s="59" t="n">
         <v>0.051</v>
       </c>
-      <c r="C23" s="37" t="n">
+      <c r="C23" s="59" t="n">
         <v>0.147</v>
       </c>
     </row>
@@ -2319,10 +2502,10 @@
           <t>Vergleichsverhandlung</t>
         </is>
       </c>
-      <c r="B24" s="39" t="n">
+      <c r="B24" s="60" t="n">
         <v>0.15</v>
       </c>
-      <c r="C24" s="39" t="n">
+      <c r="C24" s="60" t="n">
         <v>0.023</v>
       </c>
     </row>
@@ -2332,10 +2515,10 @@
           <t>Gutachten</t>
         </is>
       </c>
-      <c r="B25" s="37" t="n">
+      <c r="B25" s="59" t="n">
         <v>0.123</v>
       </c>
-      <c r="C25" s="37" t="n">
+      <c r="C25" s="59" t="n">
         <v>-0.319</v>
       </c>
     </row>
@@ -2345,10 +2528,10 @@
           <t>Unterliegensquote Kläger</t>
         </is>
       </c>
-      <c r="B26" s="39" t="n">
+      <c r="B26" s="60" t="n">
         <v>0</v>
       </c>
-      <c r="C26" s="39" t="n">
+      <c r="C26" s="60" t="n">
         <v>0.122</v>
       </c>
     </row>
@@ -2383,10 +2566,10 @@
           <t>Forderung Dienstleistungen</t>
         </is>
       </c>
-      <c r="B31" s="37" t="n">
+      <c r="B31" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="C31" s="37" t="n">
+      <c r="C31" s="59" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2396,10 +2579,10 @@
           <t>Forderung Bau</t>
         </is>
       </c>
-      <c r="B32" s="39" t="n">
+      <c r="B32" s="60" t="n">
         <v>0.037</v>
       </c>
-      <c r="C32" s="39" t="n">
+      <c r="C32" s="60" t="n">
         <v>-0.208</v>
       </c>
     </row>
@@ -2409,10 +2592,10 @@
           <t>Forderung Handel</t>
         </is>
       </c>
-      <c r="B33" s="37" t="n">
+      <c r="B33" s="59" t="n">
         <v>0.007</v>
       </c>
-      <c r="C33" s="37" t="n">
+      <c r="C33" s="59" t="n">
         <v>0.004</v>
       </c>
     </row>
@@ -2422,10 +2605,10 @@
           <t>Forderung Finanz/Versicherung</t>
         </is>
       </c>
-      <c r="B34" s="39" t="n">
+      <c r="B34" s="60" t="n">
         <v>0.068</v>
       </c>
-      <c r="C34" s="39" t="n">
+      <c r="C34" s="60" t="n">
         <v>-0.12</v>
       </c>
     </row>
@@ -2435,10 +2618,10 @@
           <t>Haftung Gesellschaftsorgane</t>
         </is>
       </c>
-      <c r="B35" s="37" t="n">
+      <c r="B35" s="59" t="n">
         <v>-0.006</v>
       </c>
-      <c r="C35" s="37" t="n">
+      <c r="C35" s="59" t="n">
         <v>-0.064</v>
       </c>
     </row>
@@ -2448,10 +2631,10 @@
           <t>UWG/URG</t>
         </is>
       </c>
-      <c r="B36" s="39" t="n">
+      <c r="B36" s="60" t="n">
         <v>0.592</v>
       </c>
-      <c r="C36" s="39" t="n">
+      <c r="C36" s="60" t="n">
         <v>1.058</v>
       </c>
     </row>
@@ -2461,10 +2644,10 @@
           <t>Immaterialgüterrecht</t>
         </is>
       </c>
-      <c r="B37" s="37" t="n">
+      <c r="B37" s="59" t="n">
         <v>0.06900000000000001</v>
       </c>
-      <c r="C37" s="37" t="n">
+      <c r="C37" s="59" t="n">
         <v>-0.079</v>
       </c>
     </row>
@@ -2474,10 +2657,10 @@
           <t>Gesellschaftsrecht</t>
         </is>
       </c>
-      <c r="B38" s="39" t="n">
+      <c r="B38" s="60" t="n">
         <v>-0.227</v>
       </c>
-      <c r="C38" s="39" t="n">
+      <c r="C38" s="60" t="n">
         <v>-0.045</v>
       </c>
     </row>
@@ -2487,10 +2670,10 @@
           <t>Übrige</t>
         </is>
       </c>
-      <c r="B39" s="37" t="n">
+      <c r="B39" s="59" t="n">
         <v>0.029</v>
       </c>
-      <c r="C39" s="37" t="n">
+      <c r="C39" s="59" t="n">
         <v>-0.159</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve disclaimer formatting in litigation cost calculator
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/publications/Litigation_Cost_Calculator_Commercial_Courts_based_on_empirical_findings.xlsx
+++ b/publications/Litigation_Cost_Calculator_Commercial_Courts_based_on_empirical_findings.xlsx
@@ -122,15 +122,15 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="11"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
       <color rgb="00FFFFFF"/>
-      <sz val="9"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -193,8 +193,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CC0000"/>
-        <bgColor rgb="00CC0000"/>
+        <fgColor rgb="008B0000"/>
+        <bgColor rgb="008B0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B22222"/>
+        <bgColor rgb="00B22222"/>
       </patternFill>
     </fill>
   </fills>
@@ -335,7 +341,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -419,11 +425,14 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="11" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -821,7 +830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C60"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -829,7 +838,7 @@
     <col width="36" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="8" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="A1" s="41" t="inlineStr">
         <is>
           <t>HAFTUNGSAUSSCHLUSS</t>
@@ -838,37 +847,33 @@
       <c r="B1" s="42" t="n"/>
       <c r="C1" s="42" t="n"/>
     </row>
-    <row r="2" ht="90" customHeight="1">
+    <row r="2" ht="20" customHeight="1">
       <c r="A2" s="43" t="inlineStr">
         <is>
           <t>Dieses Tool dient ausschliesslich zu Informations- und Bildungszwecken. Die Kostenschätzungen basieren auf statistischen Regressionsmodellen und empirischen Daten gemäss der Studie «From Tariff to Award». Die Ergebnisse sind Näherungswerte und können erheblich von den tatsächlich zugesprochenen Prozesskosten abweichen.
 Der Autor übernimmt keinerlei Haftung für die Richtigkeit, Vollständigkeit, Aktualität oder Zuverlässigkeit der mit diesem Tool generierten Schätzungen. Die Nutzung dieses Tools stellt keine Rechtsberatung dar. Es werden keinerlei Gewährleistungen abgegeben. Für fallspezifische Kosteneinschätzungen ist eine unabhängige fachkundige Beratung einzuholen.</t>
         </is>
       </c>
-      <c r="B2" s="42" t="n"/>
-      <c r="C2" s="42" t="n"/>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="42" t="n"/>
-      <c r="B3" s="42" t="n"/>
-      <c r="C3" s="42" t="n"/>
-    </row>
-    <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="42" t="n"/>
-      <c r="B4" s="42" t="n"/>
-      <c r="C4" s="42" t="n"/>
-    </row>
-    <row r="5" ht="26" customHeight="1">
-      <c r="A5" s="42" t="n"/>
-      <c r="B5" s="42" t="n"/>
-      <c r="C5" s="42" t="n"/>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="42" t="n"/>
-      <c r="B6" s="42" t="n"/>
-      <c r="C6" s="42" t="n"/>
-    </row>
-    <row r="7" ht="24" customHeight="1">
+      <c r="B2" s="44" t="n"/>
+      <c r="C2" s="44" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="44" t="n"/>
+      <c r="B3" s="44" t="n"/>
+      <c r="C3" s="44" t="n"/>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="44" t="n"/>
+      <c r="B4" s="44" t="n"/>
+      <c r="C4" s="44" t="n"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="44" t="n"/>
+      <c r="B5" s="44" t="n"/>
+      <c r="C5" s="44" t="n"/>
+    </row>
+    <row r="6" ht="6" customHeight="1"/>
+    <row r="7" ht="30" customHeight="1">
       <c r="A7" s="41" t="inlineStr">
         <is>
           <t>DISCLAIMER</t>
@@ -877,144 +882,124 @@
       <c r="B7" s="42" t="n"/>
       <c r="C7" s="42" t="n"/>
     </row>
-    <row r="8" ht="90" customHeight="1">
+    <row r="8" ht="20" customHeight="1">
       <c r="A8" s="43" t="inlineStr">
         <is>
           <t>This tool is provided for informational and educational purposes only. The cost estimates are based on statistical regression models and empirical data from the study «From Tariff to Award». The results are approximations and may differ significantly from actual litigation costs awarded by the court.
 The author assumes no liability for the accuracy, completeness, timeliness, or reliability of the estimates generated by this tool. Use of this tool does not constitute legal advice. No warranties of any kind are given. For case-specific cost assessments, independent professional advice should be sought.</t>
         </is>
       </c>
-      <c r="B8" s="42" t="n"/>
-      <c r="C8" s="42" t="n"/>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="42" t="n"/>
-      <c r="B9" s="42" t="n"/>
-      <c r="C9" s="42" t="n"/>
-    </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="42" t="n"/>
-      <c r="B10" s="42" t="n"/>
-      <c r="C10" s="42" t="n"/>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="42" t="n"/>
-      <c r="B11" s="42" t="n"/>
-      <c r="C11" s="42" t="n"/>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="42" t="n"/>
-      <c r="B12" s="42" t="n"/>
-      <c r="C12" s="42" t="n"/>
-    </row>
-    <row r="13" ht="24" customHeight="1"/>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="B8" s="44" t="n"/>
+      <c r="C8" s="44" t="n"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="44" t="n"/>
+      <c r="B9" s="44" t="n"/>
+      <c r="C9" s="44" t="n"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="44" t="n"/>
+      <c r="B10" s="44" t="n"/>
+      <c r="C10" s="44" t="n"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="44" t="n"/>
+      <c r="B11" s="44" t="n"/>
+      <c r="C11" s="44" t="n"/>
+    </row>
+    <row r="12" ht="6" customHeight="1"/>
+    <row r="13" ht="6" customHeight="1"/>
+    <row r="14" ht="18" customHeight="1"/>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>Prozesskostenrechner</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Ordentliche Verfahren vor den Handelsgerichten Zürich und Aargau — Modell 6</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Bitte füllen Sie die gelb markierten Felder aus. Die Ergebnisse werden automatisch berechnet. Das Tool schätzt Gerichtskosten (vom Gericht festgesetzt) und Parteientschädigung (Anwaltskostenersatz an die obsiegende Partei) auf Basis von über 900 Urteilen.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">   EINGABE</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Fall</t>
         </is>
       </c>
-      <c r="B18" s="7" t="n"/>
-      <c r="C18" s="7" t="n"/>
-    </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>Kanton</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>Zürich</t>
-        </is>
-      </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>Standort des zuständigen Handelsgerichts</t>
-        </is>
-      </c>
+      <c r="B19" s="7" t="n"/>
+      <c r="C19" s="7" t="n"/>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Streitwert (CHF)</t>
-        </is>
-      </c>
-      <c r="B20" s="44" t="n">
-        <v>500000</v>
+          <t>Kanton</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Gesamtwert aller Rechtsbegehren</t>
+          <t>Standort des zuständigen Handelsgerichts</t>
         </is>
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Rechtsgebiet</t>
-        </is>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>Forderung Dienstleistungen</t>
-        </is>
+          <t>Streitwert (CHF)</t>
+        </is>
+      </c>
+      <c r="B21" s="45" t="n">
+        <v>500000</v>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Hauptkategorie gemäss Urteilskopf</t>
+          <t>Gesamtwert aller Rechtsbegehren</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>Kläger mit Sitz in der Schweiz</t>
+          <t>Rechtsgebiet</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Forderung Dienstleistungen</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>Sitz oder Wohnsitz in der Schweiz?</t>
+          <t>Hauptkategorie gemäss Urteilskopf</t>
         </is>
       </c>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Beklagter mit Sitz in der Schweiz</t>
+          <t>Kläger mit Sitz in der Schweiz</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
@@ -1031,22 +1016,24 @@
     <row r="24" ht="10" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>Anzahl Kläger</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="n">
-        <v>1</v>
+          <t>Beklagter mit Sitz in der Schweiz</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>inkl. allfälliger Streitgenossen</t>
+          <t>Sitz oder Wohnsitz in der Schweiz?</t>
         </is>
       </c>
     </row>
     <row r="25" ht="26" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>Anzahl Beklagte</t>
+          <t>Anzahl Kläger</t>
         </is>
       </c>
       <c r="B25" s="9" t="n">
@@ -1059,52 +1046,50 @@
       </c>
     </row>
     <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t>Anzahl Beklagte</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>inkl. allfälliger Streitgenossen</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Verfahrensgang (erwartete oder eingetretene Prozessschritte)</t>
         </is>
       </c>
-      <c r="B26" s="7" t="n"/>
-      <c r="C26" s="7" t="n"/>
-    </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="8" t="inlineStr">
-        <is>
-          <t>Klagantwort eingereicht</t>
-        </is>
-      </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="C27" s="10" t="inlineStr">
-        <is>
-          <t>Hat der Beklagte eine Klagantwort eingereicht?</t>
-        </is>
-      </c>
+      <c r="B27" s="7" t="n"/>
+      <c r="C27" s="7" t="n"/>
     </row>
     <row r="28" ht="6" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>Zweiter Schriftenwechsel</t>
+          <t>Klagantwort eingereicht</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Nein</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Replik und Duplik angeordnet?</t>
+          <t>Hat der Beklagte eine Klagantwort eingereicht?</t>
         </is>
       </c>
     </row>
     <row r="29" ht="24" customHeight="1">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Widerklage erhoben</t>
+          <t>Zweiter Schriftenwechsel</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
@@ -1114,14 +1099,14 @@
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Hat der Beklagte eine Widerklage erhoben?</t>
+          <t>Replik und Duplik angeordnet?</t>
         </is>
       </c>
     </row>
     <row r="30" ht="24" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>Widerklage mit 2. Schriftenwechsel</t>
+          <t>Widerklage erhoben</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
@@ -1131,14 +1116,14 @@
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>Zweiter Schriftenwechsel zur Widerklage?</t>
+          <t>Hat der Beklagte eine Widerklage erhoben?</t>
         </is>
       </c>
     </row>
     <row r="31" ht="4" customHeight="1">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>Zusätzliche Eingaben</t>
+          <t>Widerklage mit 2. Schriftenwechsel</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
@@ -1148,14 +1133,14 @@
       </c>
       <c r="C31" s="10" t="inlineStr">
         <is>
-          <t>Weitere Eingaben über die Schriftenw. hinaus?</t>
+          <t>Zweiter Schriftenwechsel zur Widerklage?</t>
         </is>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>Vergleichsverhandlung</t>
+          <t>Zusätzliche Eingaben</t>
         </is>
       </c>
       <c r="B32" s="9" t="inlineStr">
@@ -1165,289 +1150,308 @@
       </c>
       <c r="C32" s="10" t="inlineStr">
         <is>
-          <t>Wurde eine Vergleichsverhandlung durchgeführt?</t>
+          <t>Weitere Eingaben über die Schriftenw. hinaus?</t>
         </is>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="8" t="inlineStr">
         <is>
+          <t>Vergleichsverhandlung</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t>Wurde eine Vergleichsverhandlung durchgeführt?</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="26" customHeight="1">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
           <t>Gutachten</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>Nein</t>
         </is>
       </c>
-      <c r="C33" s="10" t="inlineStr">
+      <c r="C34" s="10" t="inlineStr">
         <is>
           <t>Wurde ein Sachverständigengutachten eingeholt?</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="26" customHeight="1">
-      <c r="A34" s="6" t="inlineStr">
+    <row r="35" ht="26" customHeight="1">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">  Kostenverteilung</t>
         </is>
       </c>
-      <c r="B34" s="7" t="n"/>
-      <c r="C34" s="7" t="n"/>
-    </row>
-    <row r="35" ht="26" customHeight="1">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="B35" s="7" t="n"/>
+      <c r="C35" s="7" t="n"/>
+    </row>
+    <row r="36" ht="6" customHeight="1">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>Unterliegensquote Kläger (0–1)</t>
         </is>
       </c>
-      <c r="B35" s="12" t="n">
+      <c r="B36" s="12" t="n">
         <v>0.5</v>
       </c>
-      <c r="C35" s="10" t="inlineStr">
+      <c r="C36" s="10" t="inlineStr">
         <is>
           <t>0 = Kl. obsiegt, 1 = Kl. unterliegt (beeinflusst nur PE)</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="6" customHeight="1"/>
-    <row r="37" ht="24" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="37" ht="24" customHeight="1"/>
+    <row r="38" ht="24" customHeight="1">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">   ERGEBNISSE</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="24" customHeight="1">
-      <c r="A38" s="13" t="inlineStr">
+    <row r="39" ht="10" customHeight="1">
+      <c r="A39" s="13" t="inlineStr">
         <is>
           <t>Gerichtskosten gemäss Tarif</t>
         </is>
       </c>
-      <c r="B38" s="45">
+      <c r="B39" s="46">
         <f>IF(B7="Zürich",MAX(150,INDEX(Tarif!C$3:C$10,MATCH(B8,Tarif!A$3:A$10,1))+(B8-INDEX(Tarif!A$3:A$10,MATCH(B8,Tarif!A$3:A$10,1)))*INDEX(Tarif!D$3:D$10,MATCH(B8,Tarif!A$3:A$10,1))),INDEX(Tarif!C$19:C$28,MATCH(B8,Tarif!A$19:A$28,1))+B8*INDEX(Tarif!D$19:D$28,MATCH(B8,Tarif!A$19:A$28,1)))</f>
         <v/>
       </c>
-      <c r="C38" s="15" t="inlineStr">
+      <c r="C39" s="15" t="inlineStr">
         <is>
           <t>Gesetzlicher Ausgangswert (GebV OG ZH / GebT AG)</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="10" customHeight="1">
-      <c r="A39" s="13" t="inlineStr">
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="13" t="inlineStr">
         <is>
           <t>Parteientschädigung gemäss Tarif</t>
         </is>
       </c>
-      <c r="B39" s="45">
+      <c r="B40" s="46">
         <f>IF(B7="Zürich",MAX(100,INDEX(Tarif!H$3:H$14,MATCH(B8,Tarif!F$3:F$14,1))+(B8-INDEX(Tarif!F$3:F$14,MATCH(B8,Tarif!F$3:F$14,1)))*INDEX(Tarif!I$3:I$14,MATCH(B8,Tarif!F$3:F$14,1))),INDEX(Tarif!H$19:H$30,MATCH(B8,Tarif!F$19:F$30,1))+B8*INDEX(Tarif!I$19:I$30,MATCH(B8,Tarif!F$19:F$30,1)))</f>
         <v/>
       </c>
-      <c r="C39" s="15" t="inlineStr">
+      <c r="C40" s="15" t="inlineStr">
         <is>
           <t>Gesetzlicher Ausgangswert (AnwGebV ZH / AnwT AG)</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="18" customHeight="1"/>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="13" t="inlineStr">
+    <row r="41" ht="18" customHeight="1"/>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="13" t="inlineStr">
         <is>
           <t>Geschätzte Gerichtskosten</t>
         </is>
       </c>
-      <c r="B41" s="45">
+      <c r="B42" s="46">
         <f>B26*EXP(B47)</f>
         <v/>
       </c>
-      <c r="C41" s="15" t="inlineStr">
+      <c r="C42" s="15" t="inlineStr">
         <is>
           <t>Modellschätzung basierend auf 976 Urteilen</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="13" t="inlineStr">
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
         <is>
           <t>Geschätzte Parteientschädigung</t>
         </is>
       </c>
-      <c r="B42" s="45">
+      <c r="B43" s="46">
         <f>B27*EXP(B48)</f>
         <v/>
       </c>
-      <c r="C42" s="15" t="inlineStr">
+      <c r="C43" s="15" t="inlineStr">
         <is>
           <t>Modellschätzung basierend auf 898 Urteilen</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="18" customHeight="1"/>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="16" t="inlineStr">
+    <row r="44" ht="18" customHeight="1"/>
+    <row r="45" ht="16" customHeight="1">
+      <c r="A45" s="16" t="inlineStr">
         <is>
           <t>GESCHÄTZTE GESAMTKOSTEN</t>
         </is>
       </c>
-      <c r="B44" s="46">
+      <c r="B45" s="47">
         <f>B29+B30</f>
         <v/>
       </c>
-      <c r="C44" s="18" t="inlineStr">
+      <c r="C45" s="18" t="inlineStr">
         <is>
           <t>Summe GK + PE (ohne eigene Anwaltskosten)</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="16" customHeight="1">
-      <c r="A45" s="19" t="inlineStr">
+    <row r="46" ht="16" customHeight="1">
+      <c r="A46" s="19" t="inlineStr">
         <is>
           <t>Bandbreite: In 50% der Fälle liegen die tatsächlichen Kosten innerhalb dieses Bereichs.</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="16" customHeight="1">
-      <c r="A46" s="20" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="20" t="inlineStr">
         <is>
           <t>Bandbreite Gerichtskosten (±21%)</t>
         </is>
       </c>
-      <c r="B46" s="47">
+      <c r="B47" s="48">
         <f>B29*(1-0.21)</f>
         <v/>
       </c>
-      <c r="C46" s="47">
+      <c r="C47" s="48">
         <f>B29*(1+0.21)</f>
         <v/>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="20" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="20" t="inlineStr">
         <is>
           <t>Bandbreite Parteientschädigung (±25.8%)</t>
         </is>
       </c>
-      <c r="B47" s="47">
+      <c r="B48" s="48">
         <f>B30*(1-0.258)</f>
         <v/>
       </c>
-      <c r="C47" s="47">
+      <c r="C48" s="48">
         <f>B30*(1+0.258)</f>
         <v/>
       </c>
     </row>
-    <row r="48"/>
-    <row r="49">
-      <c r="A49" s="13" t="inlineStr">
+    <row r="49"/>
+    <row r="50">
+      <c r="A50" s="13" t="inlineStr">
         <is>
           <t>Abweichung vom Tarif — Gerichtskosten</t>
         </is>
       </c>
-      <c r="B49" s="48">
+      <c r="B50" s="49">
         <f>(B29-B26)/B26</f>
         <v/>
       </c>
-      <c r="C49" s="15" t="inlineStr">
+      <c r="C50" s="15" t="inlineStr">
         <is>
           <t>positiv = über Tarif, negativ = unter Tarif</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="13" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="13" t="inlineStr">
         <is>
           <t>Abweichung vom Tarif — Parteientschädigung</t>
         </is>
       </c>
-      <c r="B50" s="48">
+      <c r="B51" s="49">
         <f>(B30-B27)/B27</f>
         <v/>
       </c>
-      <c r="C50" s="15" t="inlineStr">
+      <c r="C51" s="15" t="inlineStr">
         <is>
           <t>positiv = über Tarif, negativ = unter Tarif</t>
         </is>
       </c>
     </row>
-    <row r="51"/>
-    <row r="52">
-      <c r="A52" s="23" t="inlineStr">
+    <row r="52"/>
+    <row r="53">
+      <c r="A53" s="23" t="inlineStr">
         <is>
           <t>HAFTUNGSAUSSCHLUSS: Dieses Tool dient ausschliesslich zu Informations- und Bildungszwecken. Die Kostenschätzungen basieren auf statistischen Regressionsmodellen und empirischen Daten gemäss der Studie «From Tariff to Award». Die Ergebnisse sind Näherungswerte und können erheblich von den tatsächlich zugesprochenen Prozesskosten abweichen.
 Der Autor übernimmt keinerlei Haftung für die Richtigkeit, Vollständigkeit, Aktualität oder Zuverlässigkeit der mit diesem Tool generierten Schätzungen. Die Nutzung dieses Tools stellt keine Rechtsberatung dar. Es werden keinerlei Gewährleistungen abgegeben. Für fallspezifische Kosteneinschätzungen ist eine unabhängige fachkundige Beratung einzuholen.</t>
         </is>
       </c>
-      <c r="B52" s="49" t="n"/>
-      <c r="C52" s="50" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="51" t="n"/>
-      <c r="C53" s="52" t="n"/>
+      <c r="B53" s="50" t="n"/>
+      <c r="C53" s="51" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="51" t="n"/>
-      <c r="C54" s="52" t="n"/>
+      <c r="A54" s="52" t="n"/>
+      <c r="C54" s="53" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="51" t="n"/>
-      <c r="C55" s="52" t="n"/>
+      <c r="A55" s="52" t="n"/>
+      <c r="C55" s="53" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="53" t="n"/>
-      <c r="B56" s="54" t="n"/>
-      <c r="C56" s="55" t="n"/>
+      <c r="A56" s="52" t="n"/>
+      <c r="C56" s="53" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="19" t="inlineStr">
+      <c r="A57" s="54" t="n"/>
+      <c r="B57" s="55" t="n"/>
+      <c r="C57" s="56" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="19" t="inlineStr">
         <is>
           <t>Grundlage: «From Tariff to Award» — Modell 6 (Year FE + Judge FE). Medianer abs. Prognosefehler: GK 21%, PE 25.8%.</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="25" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="25" t="inlineStr">
         <is>
           <t>HILFSBERECHNUNGEN</t>
         </is>
       </c>
-      <c r="B58" s="26" t="n"/>
-      <c r="C58" s="26" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="27" t="inlineStr">
+      <c r="B59" s="26" t="n"/>
+      <c r="C59" s="26" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="27" t="inlineStr">
         <is>
           <t>ln(GK / Grundtarif)</t>
         </is>
       </c>
-      <c r="B59" s="56">
+      <c r="B60" s="57">
         <f>Koeffizienten!B3+LN(B26)*Koeffizienten!B4+IF(B7="Aargau",1,0)*Koeffizienten!B5+IF(B7="Aargau",1,0)*LN(B26)*Koeffizienten!B6+INDEX(Koeffizienten!B$31:B$39,MATCH(B9,Koeffizienten!A$31:A$39,0))+IF(B10="Ja",1,0)*Koeffizienten!B9+IF(B11="Ja",1,0)*Koeffizienten!B10+LN(MAX(1,B12))*Koeffizienten!B7+LN(MAX(1,B13))*Koeffizienten!B8+IF(B15="Ja",1,0)*Koeffizienten!B19+IF(B16="Ja",1,0)*Koeffizienten!B20+IF(B17="Ja",1,0)*Koeffizienten!B21+IF(B18="Ja",1,0)*Koeffizienten!B22+IF(B19="Ja",1,0)*Koeffizienten!B23+IF(B20="Ja",1,0)*Koeffizienten!B24+IF(B21="Ja",1,0)*Koeffizienten!B25</f>
         <v/>
       </c>
-      <c r="C59" s="26" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="27" t="inlineStr">
+      <c r="C60" s="26" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="27" t="inlineStr">
         <is>
           <t>ln(PE / Grundtarif)</t>
         </is>
       </c>
-      <c r="B60" s="56">
+      <c r="B61" s="57">
         <f>Koeffizienten!C3+LN(B27)*Koeffizienten!C4+IF(B7="Aargau",1,0)*Koeffizienten!C5+IF(B7="Aargau",1,0)*LN(B27)*Koeffizienten!C6+INDEX(Koeffizienten!C$31:C$39,MATCH(B9,Koeffizienten!A$31:A$39,0))+IF(B10="Ja",1,0)*Koeffizienten!C9+IF(B11="Ja",1,0)*Koeffizienten!C10+LN(MAX(1,B12))*Koeffizienten!C7+LN(MAX(1,B13))*Koeffizienten!C8+IF(B15="Ja",1,0)*Koeffizienten!C19+IF(B16="Ja",1,0)*Koeffizienten!C20+IF(B17="Ja",1,0)*Koeffizienten!C21+IF(B18="Ja",1,0)*Koeffizienten!C22+IF(B19="Ja",1,0)*Koeffizienten!C23+IF(B20="Ja",1,0)*Koeffizienten!C24+IF(B21="Ja",1,0)*Koeffizienten!C25+B23*Koeffizienten!C26</f>
         <v/>
       </c>
-      <c r="C60" s="26" t="n"/>
+      <c r="C61" s="26" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="12">
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="A33:C33"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A45:C45"/>
+    <mergeCell ref="A1:C1"/>
     <mergeCell ref="A40:C44"/>
-    <mergeCell ref="A2:C6"/>
     <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A8:C12"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A8:C11"/>
+    <mergeCell ref="A2:C5"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
@@ -1561,7 +1565,7 @@
       <c r="C3" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="D3" s="57" t="n">
+      <c r="D3" s="58" t="n">
         <v>0.25</v>
       </c>
       <c r="F3" s="31" t="n">
@@ -1573,7 +1577,7 @@
       <c r="H3" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="I3" s="57" t="n">
+      <c r="I3" s="58" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -1587,7 +1591,7 @@
       <c r="C4" s="33" t="n">
         <v>250</v>
       </c>
-      <c r="D4" s="58" t="n">
+      <c r="D4" s="59" t="n">
         <v>0.2</v>
       </c>
       <c r="F4" s="33" t="n">
@@ -1599,7 +1603,7 @@
       <c r="H4" s="33" t="n">
         <v>1250</v>
       </c>
-      <c r="I4" s="58" t="n">
+      <c r="I4" s="59" t="n">
         <v>0.23</v>
       </c>
     </row>
@@ -1613,7 +1617,7 @@
       <c r="C5" s="31" t="n">
         <v>1050</v>
       </c>
-      <c r="D5" s="57" t="n">
+      <c r="D5" s="58" t="n">
         <v>0.14</v>
       </c>
       <c r="F5" s="31" t="n">
@@ -1625,7 +1629,7 @@
       <c r="H5" s="31" t="n">
         <v>2400</v>
       </c>
-      <c r="I5" s="57" t="n">
+      <c r="I5" s="58" t="n">
         <v>0.15</v>
       </c>
     </row>
@@ -1639,7 +1643,7 @@
       <c r="C6" s="33" t="n">
         <v>3150</v>
       </c>
-      <c r="D6" s="58" t="n">
+      <c r="D6" s="59" t="n">
         <v>0.08</v>
       </c>
       <c r="F6" s="33" t="n">
@@ -1651,7 +1655,7 @@
       <c r="H6" s="33" t="n">
         <v>3900</v>
       </c>
-      <c r="I6" s="58" t="n">
+      <c r="I6" s="59" t="n">
         <v>0.11</v>
       </c>
     </row>
@@ -1665,7 +1669,7 @@
       <c r="C7" s="31" t="n">
         <v>7950</v>
       </c>
-      <c r="D7" s="57" t="n">
+      <c r="D7" s="58" t="n">
         <v>0.04</v>
       </c>
       <c r="F7" s="31" t="n">
@@ -1677,7 +1681,7 @@
       <c r="H7" s="31" t="n">
         <v>6100</v>
       </c>
-      <c r="I7" s="57" t="n">
+      <c r="I7" s="58" t="n">
         <v>0.09</v>
       </c>
     </row>
@@ -1691,7 +1695,7 @@
       <c r="C8" s="33" t="n">
         <v>16750</v>
       </c>
-      <c r="D8" s="58" t="n">
+      <c r="D8" s="59" t="n">
         <v>0.02</v>
       </c>
       <c r="F8" s="33" t="n">
@@ -1703,7 +1707,7 @@
       <c r="H8" s="33" t="n">
         <v>9700</v>
       </c>
-      <c r="I8" s="58" t="n">
+      <c r="I8" s="59" t="n">
         <v>0.06</v>
       </c>
     </row>
@@ -1717,7 +1721,7 @@
       <c r="C9" s="31" t="n">
         <v>30750</v>
       </c>
-      <c r="D9" s="57" t="n">
+      <c r="D9" s="58" t="n">
         <v>0.01</v>
       </c>
       <c r="F9" s="31" t="n">
@@ -1729,7 +1733,7 @@
       <c r="H9" s="31" t="n">
         <v>14500</v>
       </c>
-      <c r="I9" s="57" t="n">
+      <c r="I9" s="58" t="n">
         <v>0.035</v>
       </c>
     </row>
@@ -1743,7 +1747,7 @@
       <c r="C10" s="33" t="n">
         <v>120750</v>
       </c>
-      <c r="D10" s="58" t="n">
+      <c r="D10" s="59" t="n">
         <v>0.005</v>
       </c>
       <c r="F10" s="33" t="n">
@@ -1755,7 +1759,7 @@
       <c r="H10" s="33" t="n">
         <v>19400</v>
       </c>
-      <c r="I10" s="58" t="n">
+      <c r="I10" s="59" t="n">
         <v>0.02</v>
       </c>
     </row>
@@ -1769,7 +1773,7 @@
       <c r="H11" s="31" t="n">
         <v>25400</v>
       </c>
-      <c r="I11" s="57" t="n">
+      <c r="I11" s="58" t="n">
         <v>0.015</v>
       </c>
     </row>
@@ -1783,7 +1787,7 @@
       <c r="H12" s="33" t="n">
         <v>31400</v>
       </c>
-      <c r="I12" s="58" t="n">
+      <c r="I12" s="59" t="n">
         <v>0.01</v>
       </c>
     </row>
@@ -1797,7 +1801,7 @@
       <c r="H13" s="31" t="n">
         <v>61400</v>
       </c>
-      <c r="I13" s="57" t="n">
+      <c r="I13" s="58" t="n">
         <v>0.0075</v>
       </c>
     </row>
@@ -1811,7 +1815,7 @@
       <c r="H14" s="33" t="n">
         <v>106400</v>
       </c>
-      <c r="I14" s="58" t="n">
+      <c r="I14" s="59" t="n">
         <v>0.005</v>
       </c>
     </row>
@@ -1879,7 +1883,7 @@
       <c r="C19" s="31" t="n">
         <v>900</v>
       </c>
-      <c r="D19" s="57" t="n">
+      <c r="D19" s="58" t="n">
         <v>0.11</v>
       </c>
       <c r="F19" s="31" t="n">
@@ -1891,7 +1895,7 @@
       <c r="H19" s="31" t="n">
         <v>1110</v>
       </c>
-      <c r="I19" s="57" t="n">
+      <c r="I19" s="58" t="n">
         <v>0.22</v>
       </c>
     </row>
@@ -1905,7 +1909,7 @@
       <c r="C20" s="33" t="n">
         <v>1160</v>
       </c>
-      <c r="D20" s="58" t="n">
+      <c r="D20" s="59" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="F20" s="33" t="n">
@@ -1917,7 +1921,7 @@
       <c r="H20" s="33" t="n">
         <v>1230</v>
       </c>
-      <c r="I20" s="58" t="n">
+      <c r="I20" s="59" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1931,7 +1935,7 @@
       <c r="C21" s="31" t="n">
         <v>1290</v>
       </c>
-      <c r="D21" s="57" t="n">
+      <c r="D21" s="58" t="n">
         <v>0.06</v>
       </c>
       <c r="F21" s="31" t="n">
@@ -1943,7 +1947,7 @@
       <c r="H21" s="31" t="n">
         <v>1850</v>
       </c>
-      <c r="I21" s="57" t="n">
+      <c r="I21" s="58" t="n">
         <v>0.15</v>
       </c>
     </row>
@@ -1957,7 +1961,7 @@
       <c r="C22" s="33" t="n">
         <v>770</v>
       </c>
-      <c r="D22" s="58" t="n">
+      <c r="D22" s="59" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="F22" s="33" t="n">
@@ -1969,7 +1973,7 @@
       <c r="H22" s="33" t="n">
         <v>2590</v>
       </c>
-      <c r="I22" s="58" t="n">
+      <c r="I22" s="59" t="n">
         <v>0.12</v>
       </c>
     </row>
@@ -1983,7 +1987,7 @@
       <c r="C23" s="31" t="n">
         <v>4270</v>
       </c>
-      <c r="D23" s="57" t="n">
+      <c r="D23" s="58" t="n">
         <v>0.035</v>
       </c>
       <c r="F23" s="31" t="n">
@@ -1995,7 +1999,7 @@
       <c r="H23" s="31" t="n">
         <v>4070</v>
       </c>
-      <c r="I23" s="57" t="n">
+      <c r="I23" s="58" t="n">
         <v>0.09</v>
       </c>
     </row>
@@ -2009,7 +2013,7 @@
       <c r="C24" s="33" t="n">
         <v>6870</v>
       </c>
-      <c r="D24" s="58" t="n">
+      <c r="D24" s="59" t="n">
         <v>0.022</v>
       </c>
       <c r="F24" s="33" t="n">
@@ -2021,7 +2025,7 @@
       <c r="H24" s="33" t="n">
         <v>6530</v>
       </c>
-      <c r="I24" s="58" t="n">
+      <c r="I24" s="59" t="n">
         <v>0.064</v>
       </c>
     </row>
@@ -2035,7 +2039,7 @@
       <c r="C25" s="31" t="n">
         <v>9670</v>
       </c>
-      <c r="D25" s="57" t="n">
+      <c r="D25" s="58" t="n">
         <v>0.015</v>
       </c>
       <c r="F25" s="31" t="n">
@@ -2047,7 +2051,7 @@
       <c r="H25" s="31" t="n">
         <v>10230</v>
       </c>
-      <c r="I25" s="57" t="n">
+      <c r="I25" s="58" t="n">
         <v>0.044</v>
       </c>
     </row>
@@ -2061,7 +2065,7 @@
       <c r="C26" s="33" t="n">
         <v>13670</v>
       </c>
-      <c r="D26" s="58" t="n">
+      <c r="D26" s="59" t="n">
         <v>0.01</v>
       </c>
       <c r="F26" s="33" t="n">
@@ -2073,7 +2077,7 @@
       <c r="H26" s="33" t="n">
         <v>14300</v>
       </c>
-      <c r="I26" s="58" t="n">
+      <c r="I26" s="59" t="n">
         <v>0.033</v>
       </c>
     </row>
@@ -2087,7 +2091,7 @@
       <c r="C27" s="31" t="n">
         <v>21670</v>
       </c>
-      <c r="D27" s="57" t="n">
+      <c r="D27" s="58" t="n">
         <v>0.005</v>
       </c>
       <c r="F27" s="31" t="n">
@@ -2099,7 +2103,7 @@
       <c r="H27" s="31" t="n">
         <v>20240</v>
       </c>
-      <c r="I27" s="57" t="n">
+      <c r="I27" s="58" t="n">
         <v>0.025</v>
       </c>
     </row>
@@ -2113,7 +2117,7 @@
       <c r="C28" s="33" t="n">
         <v>28270</v>
       </c>
-      <c r="D28" s="58" t="n">
+      <c r="D28" s="59" t="n">
         <v>0.003</v>
       </c>
       <c r="F28" s="33" t="n">
@@ -2125,7 +2129,7 @@
       <c r="H28" s="33" t="n">
         <v>29040</v>
       </c>
-      <c r="I28" s="58" t="n">
+      <c r="I28" s="59" t="n">
         <v>0.019</v>
       </c>
     </row>
@@ -2139,7 +2143,7 @@
       <c r="H29" s="31" t="n">
         <v>44440</v>
       </c>
-      <c r="I29" s="57" t="n">
+      <c r="I29" s="58" t="n">
         <v>0.014</v>
       </c>
     </row>
@@ -2153,7 +2157,7 @@
       <c r="H30" s="33" t="n">
         <v>69080</v>
       </c>
-      <c r="I30" s="58" t="n">
+      <c r="I30" s="59" t="n">
         <v>0.01</v>
       </c>
     </row>
@@ -2229,10 +2233,10 @@
           <t>Intercept</t>
         </is>
       </c>
-      <c r="B3" s="59" t="n">
+      <c r="B3" s="60" t="n">
         <v>0.927</v>
       </c>
-      <c r="C3" s="59" t="n">
+      <c r="C3" s="60" t="n">
         <v>1.888</v>
       </c>
     </row>
@@ -2242,10 +2246,10 @@
           <t>ln(Baseline)</t>
         </is>
       </c>
-      <c r="B4" s="60" t="n">
+      <c r="B4" s="61" t="n">
         <v>-0.111</v>
       </c>
-      <c r="C4" s="60" t="n">
+      <c r="C4" s="61" t="n">
         <v>-0.17</v>
       </c>
     </row>
@@ -2255,10 +2259,10 @@
           <t>D_AG</t>
         </is>
       </c>
-      <c r="B5" s="59" t="n">
+      <c r="B5" s="60" t="n">
         <v>-0.518</v>
       </c>
-      <c r="C5" s="59" t="n">
+      <c r="C5" s="60" t="n">
         <v>-3.414</v>
       </c>
     </row>
@@ -2268,10 +2272,10 @@
           <t>D_AG x ln(Baseline)</t>
         </is>
       </c>
-      <c r="B6" s="60" t="n">
+      <c r="B6" s="61" t="n">
         <v>0.057</v>
       </c>
-      <c r="C6" s="60" t="n">
+      <c r="C6" s="61" t="n">
         <v>0.463</v>
       </c>
     </row>
@@ -2281,10 +2285,10 @@
           <t>ln(Kläger)</t>
         </is>
       </c>
-      <c r="B7" s="59" t="n">
+      <c r="B7" s="60" t="n">
         <v>0.052</v>
       </c>
-      <c r="C7" s="59" t="n">
+      <c r="C7" s="60" t="n">
         <v>-0.13</v>
       </c>
     </row>
@@ -2294,10 +2298,10 @@
           <t>ln(Beklagte)</t>
         </is>
       </c>
-      <c r="B8" s="60" t="n">
+      <c r="B8" s="61" t="n">
         <v>0.092</v>
       </c>
-      <c r="C8" s="60" t="n">
+      <c r="C8" s="61" t="n">
         <v>0.176</v>
       </c>
     </row>
@@ -2307,10 +2311,10 @@
           <t>Domizil Kläger</t>
         </is>
       </c>
-      <c r="B9" s="59" t="n">
+      <c r="B9" s="60" t="n">
         <v>-0.08599999999999999</v>
       </c>
-      <c r="C9" s="59" t="n">
+      <c r="C9" s="60" t="n">
         <v>-0.129</v>
       </c>
     </row>
@@ -2320,10 +2324,10 @@
           <t>Domizil Beklagter</t>
         </is>
       </c>
-      <c r="B10" s="60" t="n">
+      <c r="B10" s="61" t="n">
         <v>-0.079</v>
       </c>
-      <c r="C10" s="60" t="n">
+      <c r="C10" s="61" t="n">
         <v>-0.022</v>
       </c>
     </row>
@@ -2333,10 +2337,10 @@
           <t>D_Bau</t>
         </is>
       </c>
-      <c r="B11" s="59" t="n">
+      <c r="B11" s="60" t="n">
         <v>0.037</v>
       </c>
-      <c r="C11" s="59" t="n">
+      <c r="C11" s="60" t="n">
         <v>-0.208</v>
       </c>
     </row>
@@ -2346,10 +2350,10 @@
           <t>D_Handel</t>
         </is>
       </c>
-      <c r="B12" s="60" t="n">
+      <c r="B12" s="61" t="n">
         <v>0.007</v>
       </c>
-      <c r="C12" s="60" t="n">
+      <c r="C12" s="61" t="n">
         <v>0.004</v>
       </c>
     </row>
@@ -2359,10 +2363,10 @@
           <t>D_Finanz/Versicherung</t>
         </is>
       </c>
-      <c r="B13" s="59" t="n">
+      <c r="B13" s="60" t="n">
         <v>0.068</v>
       </c>
-      <c r="C13" s="59" t="n">
+      <c r="C13" s="60" t="n">
         <v>-0.12</v>
       </c>
     </row>
@@ -2372,10 +2376,10 @@
           <t>D_Organhaftung</t>
         </is>
       </c>
-      <c r="B14" s="60" t="n">
+      <c r="B14" s="61" t="n">
         <v>-0.006</v>
       </c>
-      <c r="C14" s="60" t="n">
+      <c r="C14" s="61" t="n">
         <v>-0.064</v>
       </c>
     </row>
@@ -2385,10 +2389,10 @@
           <t>D_UWG/URG</t>
         </is>
       </c>
-      <c r="B15" s="59" t="n">
+      <c r="B15" s="60" t="n">
         <v>0.592</v>
       </c>
-      <c r="C15" s="59" t="n">
+      <c r="C15" s="60" t="n">
         <v>1.058</v>
       </c>
     </row>
@@ -2398,10 +2402,10 @@
           <t>D_Immaterialgüterrecht</t>
         </is>
       </c>
-      <c r="B16" s="60" t="n">
+      <c r="B16" s="61" t="n">
         <v>0.06900000000000001</v>
       </c>
-      <c r="C16" s="60" t="n">
+      <c r="C16" s="61" t="n">
         <v>-0.079</v>
       </c>
     </row>
@@ -2411,10 +2415,10 @@
           <t>D_Gesellschaftsrecht</t>
         </is>
       </c>
-      <c r="B17" s="59" t="n">
+      <c r="B17" s="60" t="n">
         <v>-0.227</v>
       </c>
-      <c r="C17" s="59" t="n">
+      <c r="C17" s="60" t="n">
         <v>-0.045</v>
       </c>
     </row>
@@ -2424,10 +2428,10 @@
           <t>D_Übrige</t>
         </is>
       </c>
-      <c r="B18" s="60" t="n">
+      <c r="B18" s="61" t="n">
         <v>0.029</v>
       </c>
-      <c r="C18" s="60" t="n">
+      <c r="C18" s="61" t="n">
         <v>-0.159</v>
       </c>
     </row>
@@ -2437,10 +2441,10 @@
           <t>Klagantwort</t>
         </is>
       </c>
-      <c r="B19" s="59" t="n">
+      <c r="B19" s="60" t="n">
         <v>-0.08799999999999999</v>
       </c>
-      <c r="C19" s="59" t="n">
+      <c r="C19" s="60" t="n">
         <v>-0.004</v>
       </c>
     </row>
@@ -2450,10 +2454,10 @@
           <t>Zweiter Schriftenwechsel</t>
         </is>
       </c>
-      <c r="B20" s="60" t="n">
+      <c r="B20" s="61" t="n">
         <v>0.504</v>
       </c>
-      <c r="C20" s="60" t="n">
+      <c r="C20" s="61" t="n">
         <v>0.319</v>
       </c>
     </row>
@@ -2463,10 +2467,10 @@
           <t>Widerklage</t>
         </is>
       </c>
-      <c r="B21" s="59" t="n">
+      <c r="B21" s="60" t="n">
         <v>-0.159</v>
       </c>
-      <c r="C21" s="59" t="n">
+      <c r="C21" s="60" t="n">
         <v>-0.173</v>
       </c>
     </row>
@@ -2476,10 +2480,10 @@
           <t>Widerklage 2. SW</t>
         </is>
       </c>
-      <c r="B22" s="60" t="n">
+      <c r="B22" s="61" t="n">
         <v>0.395</v>
       </c>
-      <c r="C22" s="60" t="n">
+      <c r="C22" s="61" t="n">
         <v>0.192</v>
       </c>
     </row>
@@ -2489,10 +2493,10 @@
           <t>Zusätzliche Eingaben</t>
         </is>
       </c>
-      <c r="B23" s="59" t="n">
+      <c r="B23" s="60" t="n">
         <v>0.051</v>
       </c>
-      <c r="C23" s="59" t="n">
+      <c r="C23" s="60" t="n">
         <v>0.147</v>
       </c>
     </row>
@@ -2502,10 +2506,10 @@
           <t>Vergleichsverhandlung</t>
         </is>
       </c>
-      <c r="B24" s="60" t="n">
+      <c r="B24" s="61" t="n">
         <v>0.15</v>
       </c>
-      <c r="C24" s="60" t="n">
+      <c r="C24" s="61" t="n">
         <v>0.023</v>
       </c>
     </row>
@@ -2515,10 +2519,10 @@
           <t>Gutachten</t>
         </is>
       </c>
-      <c r="B25" s="59" t="n">
+      <c r="B25" s="60" t="n">
         <v>0.123</v>
       </c>
-      <c r="C25" s="59" t="n">
+      <c r="C25" s="60" t="n">
         <v>-0.319</v>
       </c>
     </row>
@@ -2528,10 +2532,10 @@
           <t>Unterliegensquote Kläger</t>
         </is>
       </c>
-      <c r="B26" s="60" t="n">
+      <c r="B26" s="61" t="n">
         <v>0</v>
       </c>
-      <c r="C26" s="60" t="n">
+      <c r="C26" s="61" t="n">
         <v>0.122</v>
       </c>
     </row>
@@ -2566,10 +2570,10 @@
           <t>Forderung Dienstleistungen</t>
         </is>
       </c>
-      <c r="B31" s="59" t="n">
+      <c r="B31" s="60" t="n">
         <v>0</v>
       </c>
-      <c r="C31" s="59" t="n">
+      <c r="C31" s="60" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2579,10 +2583,10 @@
           <t>Forderung Bau</t>
         </is>
       </c>
-      <c r="B32" s="60" t="n">
+      <c r="B32" s="61" t="n">
         <v>0.037</v>
       </c>
-      <c r="C32" s="60" t="n">
+      <c r="C32" s="61" t="n">
         <v>-0.208</v>
       </c>
     </row>
@@ -2592,10 +2596,10 @@
           <t>Forderung Handel</t>
         </is>
       </c>
-      <c r="B33" s="59" t="n">
+      <c r="B33" s="60" t="n">
         <v>0.007</v>
       </c>
-      <c r="C33" s="59" t="n">
+      <c r="C33" s="60" t="n">
         <v>0.004</v>
       </c>
     </row>
@@ -2605,10 +2609,10 @@
           <t>Forderung Finanz/Versicherung</t>
         </is>
       </c>
-      <c r="B34" s="60" t="n">
+      <c r="B34" s="61" t="n">
         <v>0.068</v>
       </c>
-      <c r="C34" s="60" t="n">
+      <c r="C34" s="61" t="n">
         <v>-0.12</v>
       </c>
     </row>
@@ -2618,10 +2622,10 @@
           <t>Haftung Gesellschaftsorgane</t>
         </is>
       </c>
-      <c r="B35" s="59" t="n">
+      <c r="B35" s="60" t="n">
         <v>-0.006</v>
       </c>
-      <c r="C35" s="59" t="n">
+      <c r="C35" s="60" t="n">
         <v>-0.064</v>
       </c>
     </row>
@@ -2631,10 +2635,10 @@
           <t>UWG/URG</t>
         </is>
       </c>
-      <c r="B36" s="60" t="n">
+      <c r="B36" s="61" t="n">
         <v>0.592</v>
       </c>
-      <c r="C36" s="60" t="n">
+      <c r="C36" s="61" t="n">
         <v>1.058</v>
       </c>
     </row>
@@ -2644,10 +2648,10 @@
           <t>Immaterialgüterrecht</t>
         </is>
       </c>
-      <c r="B37" s="59" t="n">
+      <c r="B37" s="60" t="n">
         <v>0.06900000000000001</v>
       </c>
-      <c r="C37" s="59" t="n">
+      <c r="C37" s="60" t="n">
         <v>-0.079</v>
       </c>
     </row>
@@ -2657,10 +2661,10 @@
           <t>Gesellschaftsrecht</t>
         </is>
       </c>
-      <c r="B38" s="60" t="n">
+      <c r="B38" s="61" t="n">
         <v>-0.227</v>
       </c>
-      <c r="C38" s="60" t="n">
+      <c r="C38" s="61" t="n">
         <v>-0.045</v>
       </c>
     </row>
@@ -2670,10 +2674,10 @@
           <t>Übrige</t>
         </is>
       </c>
-      <c r="B39" s="59" t="n">
+      <c r="B39" s="60" t="n">
         <v>0.029</v>
       </c>
-      <c r="C39" s="59" t="n">
+      <c r="C39" s="60" t="n">
         <v>-0.159</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix litigation cost calculator: disclaimer as separate tab, all formulas intact
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/publications/Litigation_Cost_Calculator_Commercial_Courts_based_on_empirical_findings.xlsx
+++ b/publications/Litigation_Cost_Calculator_Commercial_Courts_based_on_empirical_findings.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rechner" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarif" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Koeffizienten" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Disclaimer" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rechner" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tarif" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Koeffizienten" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -119,15 +120,15 @@
       <sz val="8"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="13"/>
+      <sz val="14"/>
     </font>
     <font>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="13">
@@ -341,7 +342,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -428,7 +429,6 @@
     <xf numFmtId="0" fontId="16" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -826,11 +826,67 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="90" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="41" t="inlineStr">
+        <is>
+          <t>HAFTUNGSAUSSCHLUSS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="130" customHeight="1">
+      <c r="A2" s="42" t="inlineStr">
+        <is>
+          <t>Dieses Tool dient ausschliesslich zu Informations- und Bildungszwecken. Die Kostenschätzungen basieren auf statistischen Regressionsmodellen und empirischen Daten gemäss der Studie «From Tariff to Award». Die Ergebnisse sind Näherungswerte und können erheblich von den tatsächlich zugesprochenen Prozesskosten abweichen.
+Der Autor übernimmt keinerlei Haftung für die Richtigkeit, Vollständigkeit, Aktualität oder Zuverlässigkeit der mit diesem Tool generierten Schätzungen. Die Nutzung dieses Tools stellt keine Rechtsberatung dar. Es werden keinerlei Gewährleistungen abgegeben. Für fallspezifische Kosteneinschätzungen ist eine unabhängige fachkundige Beratung einzuholen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="43" t="n"/>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="41" t="inlineStr">
+        <is>
+          <t>DISCLAIMER</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="130" customHeight="1">
+      <c r="A5" s="42" t="inlineStr">
+        <is>
+          <t>This tool is provided for informational and educational purposes only. The cost estimates are based on statistical regression models and empirical data from the study «From Tariff to Award». The results are approximations and may differ significantly from actual litigation costs awarded by the court.
+The author assumes no liability for the accuracy, completeness, timeliness, or reliability of the estimates generated by this tool. Use of this tool does not constitute legal advice. No warranties of any kind are given. For case-specific cost assessments, independent professional advice should be sought.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="43" t="n"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="43" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="00BF8F00"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C61"/>
+  <dimension ref="A2:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -838,620 +894,545 @@
     <col width="36" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="41" t="inlineStr">
-        <is>
-          <t>HAFTUNGSAUSSCHLUSS</t>
-        </is>
-      </c>
-      <c r="B1" s="42" t="n"/>
-      <c r="C1" s="42" t="n"/>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="43" t="inlineStr">
-        <is>
-          <t>Dieses Tool dient ausschliesslich zu Informations- und Bildungszwecken. Die Kostenschätzungen basieren auf statistischen Regressionsmodellen und empirischen Daten gemäss der Studie «From Tariff to Award». Die Ergebnisse sind Näherungswerte und können erheblich von den tatsächlich zugesprochenen Prozesskosten abweichen.
-Der Autor übernimmt keinerlei Haftung für die Richtigkeit, Vollständigkeit, Aktualität oder Zuverlässigkeit der mit diesem Tool generierten Schätzungen. Die Nutzung dieses Tools stellt keine Rechtsberatung dar. Es werden keinerlei Gewährleistungen abgegeben. Für fallspezifische Kosteneinschätzungen ist eine unabhängige fachkundige Beratung einzuholen.</t>
-        </is>
-      </c>
-      <c r="B2" s="44" t="n"/>
-      <c r="C2" s="44" t="n"/>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="44" t="n"/>
-      <c r="B3" s="44" t="n"/>
-      <c r="C3" s="44" t="n"/>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="44" t="n"/>
-      <c r="B4" s="44" t="n"/>
-      <c r="C4" s="44" t="n"/>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="44" t="n"/>
-      <c r="B5" s="44" t="n"/>
-      <c r="C5" s="44" t="n"/>
-    </row>
-    <row r="6" ht="6" customHeight="1"/>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="41" t="inlineStr">
-        <is>
-          <t>DISCLAIMER</t>
-        </is>
-      </c>
-      <c r="B7" s="42" t="n"/>
-      <c r="C7" s="42" t="n"/>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="43" t="inlineStr">
-        <is>
-          <t>This tool is provided for informational and educational purposes only. The cost estimates are based on statistical regression models and empirical data from the study «From Tariff to Award». The results are approximations and may differ significantly from actual litigation costs awarded by the court.
-The author assumes no liability for the accuracy, completeness, timeliness, or reliability of the estimates generated by this tool. Use of this tool does not constitute legal advice. No warranties of any kind are given. For case-specific cost assessments, independent professional advice should be sought.</t>
-        </is>
-      </c>
-      <c r="B8" s="44" t="n"/>
-      <c r="C8" s="44" t="n"/>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="44" t="n"/>
-      <c r="B9" s="44" t="n"/>
-      <c r="C9" s="44" t="n"/>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="44" t="n"/>
-      <c r="B10" s="44" t="n"/>
-      <c r="C10" s="44" t="n"/>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="44" t="n"/>
-      <c r="B11" s="44" t="n"/>
-      <c r="C11" s="44" t="n"/>
-    </row>
-    <row r="12" ht="6" customHeight="1"/>
-    <row r="13" ht="6" customHeight="1"/>
-    <row r="14" ht="18" customHeight="1"/>
+    <row r="1" ht="8" customHeight="1"/>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Prozesskostenrechner</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Ordentliche Verfahren vor den Handelsgerichten Zürich und Aargau — Modell 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Bitte füllen Sie die gelb markierten Felder aus. Die Ergebnisse werden automatisch berechnet. Das Tool schätzt Gerichtskosten (vom Gericht festgesetzt) und Parteientschädigung (Anwaltskostenersatz an die obsiegende Partei) auf Basis von über 900 Urteilen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="26" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   EINGABE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Fall</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n"/>
+      <c r="C6" s="7" t="n"/>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Kanton</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Zürich</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Standort des zuständigen Handelsgerichts</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Streitwert (CHF)</t>
+        </is>
+      </c>
+      <c r="B8" s="44" t="n">
+        <v>500000</v>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Gesamtwert aller Rechtsbegehren</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Rechtsgebiet</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Forderung Dienstleistungen</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Hauptkategorie gemäss Urteilskopf</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Kläger mit Sitz in der Schweiz</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>Sitz oder Wohnsitz in der Schweiz?</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Beklagter mit Sitz in der Schweiz</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>Sitz oder Wohnsitz in der Schweiz?</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Anzahl Kläger</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>inkl. allfälliger Streitgenossen</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Anzahl Beklagte</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>inkl. allfälliger Streitgenossen</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Verfahrensgang (erwartete oder eingetretene Prozessschritte)</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n"/>
+    </row>
     <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>Prozesskostenrechner</t>
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Klagantwort eingereicht</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Hat der Beklagte eine Klagantwort eingereicht?</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Ordentliche Verfahren vor den Handelsgerichten Zürich und Aargau — Modell 6</t>
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Zweiter Schriftenwechsel</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>Replik und Duplik angeordnet?</t>
         </is>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Bitte füllen Sie die gelb markierten Felder aus. Die Ergebnisse werden automatisch berechnet. Das Tool schätzt Gerichtskosten (vom Gericht festgesetzt) und Parteientschädigung (Anwaltskostenersatz an die obsiegende Partei) auf Basis von über 900 Urteilen.</t>
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Widerklage erhoben</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Hat der Beklagte eine Widerklage erhoben?</t>
         </is>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   EINGABE</t>
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Widerklage mit 2. Schriftenwechsel</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Zweiter Schriftenwechsel zur Widerklage?</t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Fall</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="n"/>
-      <c r="C19" s="7" t="n"/>
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Zusätzliche Eingaben</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Weitere Eingaben über die Schriftenw. hinaus?</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Kanton</t>
+          <t>Vergleichsverhandlung</t>
         </is>
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>Zürich</t>
+          <t>Nein</t>
         </is>
       </c>
       <c r="C20" s="10" t="inlineStr">
         <is>
-          <t>Standort des zuständigen Handelsgerichts</t>
+          <t>Wurde eine Vergleichsverhandlung durchgeführt?</t>
         </is>
       </c>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Streitwert (CHF)</t>
-        </is>
-      </c>
-      <c r="B21" s="45" t="n">
-        <v>500000</v>
+          <t>Gutachten</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Gesamtwert aller Rechtsbegehren</t>
+          <t>Wurde ein Sachverständigengutachten eingeholt?</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>Rechtsgebiet</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>Forderung Dienstleistungen</t>
-        </is>
-      </c>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>Hauptkategorie gemäss Urteilskopf</t>
-        </is>
-      </c>
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Kostenverteilung</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="n"/>
+      <c r="C22" s="7" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Kläger mit Sitz in der Schweiz</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
+          <t>Unterliegensquote Kläger (0–1)</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="n">
+        <v>0.5</v>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>Sitz oder Wohnsitz in der Schweiz?</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="10" customHeight="1">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>Beklagter mit Sitz in der Schweiz</t>
-        </is>
-      </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="C24" s="10" t="inlineStr">
-        <is>
-          <t>Sitz oder Wohnsitz in der Schweiz?</t>
-        </is>
-      </c>
-    </row>
+          <t>0 = Kl. obsiegt, 1 = Kl. unterliegt (beeinflusst nur PE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="10" customHeight="1"/>
     <row r="25" ht="26" customHeight="1">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>Anzahl Kläger</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" s="10" t="inlineStr">
-        <is>
-          <t>inkl. allfälliger Streitgenossen</t>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ERGEBNISSE</t>
         </is>
       </c>
     </row>
     <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t>Anzahl Beklagte</t>
-        </is>
-      </c>
-      <c r="B26" s="9" t="n">
-        <v>1</v>
-      </c>
-      <c r="C26" s="10" t="inlineStr">
-        <is>
-          <t>inkl. allfälliger Streitgenossen</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Verfahrensgang (erwartete oder eingetretene Prozessschritte)</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="n"/>
-      <c r="C27" s="7" t="n"/>
-    </row>
-    <row r="28" ht="6" customHeight="1">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>Klagantwort eingereicht</t>
-        </is>
-      </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>Ja</t>
-        </is>
-      </c>
-      <c r="C28" s="10" t="inlineStr">
-        <is>
-          <t>Hat der Beklagte eine Klagantwort eingereicht?</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="8" t="inlineStr">
-        <is>
-          <t>Zweiter Schriftenwechsel</t>
-        </is>
-      </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>Nein</t>
-        </is>
-      </c>
-      <c r="C29" s="10" t="inlineStr">
-        <is>
-          <t>Replik und Duplik angeordnet?</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="24" customHeight="1">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>Widerklage erhoben</t>
-        </is>
-      </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>Nein</t>
-        </is>
-      </c>
-      <c r="C30" s="10" t="inlineStr">
-        <is>
-          <t>Hat der Beklagte eine Widerklage erhoben?</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="4" customHeight="1">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>Widerklage mit 2. Schriftenwechsel</t>
-        </is>
-      </c>
-      <c r="B31" s="9" t="inlineStr">
-        <is>
-          <t>Nein</t>
-        </is>
-      </c>
-      <c r="C31" s="10" t="inlineStr">
-        <is>
-          <t>Zweiter Schriftenwechsel zur Widerklage?</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="30" customHeight="1">
-      <c r="A32" s="8" t="inlineStr">
-        <is>
-          <t>Zusätzliche Eingaben</t>
-        </is>
-      </c>
-      <c r="B32" s="9" t="inlineStr">
-        <is>
-          <t>Nein</t>
-        </is>
-      </c>
-      <c r="C32" s="10" t="inlineStr">
-        <is>
-          <t>Weitere Eingaben über die Schriftenw. hinaus?</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="8" t="inlineStr">
-        <is>
-          <t>Vergleichsverhandlung</t>
-        </is>
-      </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>Nein</t>
-        </is>
-      </c>
-      <c r="C33" s="10" t="inlineStr">
-        <is>
-          <t>Wurde eine Vergleichsverhandlung durchgeführt?</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="26" customHeight="1">
-      <c r="A34" s="8" t="inlineStr">
-        <is>
-          <t>Gutachten</t>
-        </is>
-      </c>
-      <c r="B34" s="9" t="inlineStr">
-        <is>
-          <t>Nein</t>
-        </is>
-      </c>
-      <c r="C34" s="10" t="inlineStr">
-        <is>
-          <t>Wurde ein Sachverständigengutachten eingeholt?</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="26" customHeight="1">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Kostenverteilung</t>
-        </is>
-      </c>
-      <c r="B35" s="7" t="n"/>
-      <c r="C35" s="7" t="n"/>
-    </row>
-    <row r="36" ht="6" customHeight="1">
-      <c r="A36" s="8" t="inlineStr">
-        <is>
-          <t>Unterliegensquote Kläger (0–1)</t>
-        </is>
-      </c>
-      <c r="B36" s="12" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C36" s="10" t="inlineStr">
-        <is>
-          <t>0 = Kl. obsiegt, 1 = Kl. unterliegt (beeinflusst nur PE)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="24" customHeight="1"/>
-    <row r="38" ht="24" customHeight="1">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   ERGEBNISSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="10" customHeight="1">
-      <c r="A39" s="13" t="inlineStr">
+      <c r="A26" s="13" t="inlineStr">
         <is>
           <t>Gerichtskosten gemäss Tarif</t>
         </is>
       </c>
-      <c r="B39" s="46">
+      <c r="B26" s="45">
         <f>IF(B7="Zürich",MAX(150,INDEX(Tarif!C$3:C$10,MATCH(B8,Tarif!A$3:A$10,1))+(B8-INDEX(Tarif!A$3:A$10,MATCH(B8,Tarif!A$3:A$10,1)))*INDEX(Tarif!D$3:D$10,MATCH(B8,Tarif!A$3:A$10,1))),INDEX(Tarif!C$19:C$28,MATCH(B8,Tarif!A$19:A$28,1))+B8*INDEX(Tarif!D$19:D$28,MATCH(B8,Tarif!A$19:A$28,1)))</f>
         <v/>
       </c>
-      <c r="C39" s="15" t="inlineStr">
+      <c r="C26" s="15" t="inlineStr">
         <is>
           <t>Gesetzlicher Ausgangswert (GebV OG ZH / GebT AG)</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="13" t="inlineStr">
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>Parteientschädigung gemäss Tarif</t>
         </is>
       </c>
-      <c r="B40" s="46">
+      <c r="B27" s="45">
         <f>IF(B7="Zürich",MAX(100,INDEX(Tarif!H$3:H$14,MATCH(B8,Tarif!F$3:F$14,1))+(B8-INDEX(Tarif!F$3:F$14,MATCH(B8,Tarif!F$3:F$14,1)))*INDEX(Tarif!I$3:I$14,MATCH(B8,Tarif!F$3:F$14,1))),INDEX(Tarif!H$19:H$30,MATCH(B8,Tarif!F$19:F$30,1))+B8*INDEX(Tarif!I$19:I$30,MATCH(B8,Tarif!F$19:F$30,1)))</f>
         <v/>
       </c>
-      <c r="C40" s="15" t="inlineStr">
+      <c r="C27" s="15" t="inlineStr">
         <is>
           <t>Gesetzlicher Ausgangswert (AnwGebV ZH / AnwT AG)</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="18" customHeight="1"/>
-    <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="13" t="inlineStr">
+    <row r="28" ht="6" customHeight="1"/>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="13" t="inlineStr">
         <is>
           <t>Geschätzte Gerichtskosten</t>
         </is>
       </c>
-      <c r="B42" s="46">
+      <c r="B29" s="45">
         <f>B26*EXP(B47)</f>
         <v/>
       </c>
-      <c r="C42" s="15" t="inlineStr">
+      <c r="C29" s="15" t="inlineStr">
         <is>
           <t>Modellschätzung basierend auf 976 Urteilen</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="13" t="inlineStr">
+    <row r="30" ht="24" customHeight="1">
+      <c r="A30" s="13" t="inlineStr">
         <is>
           <t>Geschätzte Parteientschädigung</t>
         </is>
       </c>
-      <c r="B43" s="46">
+      <c r="B30" s="45">
         <f>B27*EXP(B48)</f>
         <v/>
       </c>
-      <c r="C43" s="15" t="inlineStr">
+      <c r="C30" s="15" t="inlineStr">
         <is>
           <t>Modellschätzung basierend auf 898 Urteilen</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="18" customHeight="1"/>
-    <row r="45" ht="16" customHeight="1">
-      <c r="A45" s="16" t="inlineStr">
+    <row r="31" ht="4" customHeight="1"/>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>GESCHÄTZTE GESAMTKOSTEN</t>
         </is>
       </c>
-      <c r="B45" s="47">
+      <c r="B32" s="46">
         <f>B29+B30</f>
         <v/>
       </c>
-      <c r="C45" s="18" t="inlineStr">
+      <c r="C32" s="18" t="inlineStr">
         <is>
           <t>Summe GK + PE (ohne eigene Anwaltskosten)</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="16" customHeight="1">
-      <c r="A46" s="19" t="inlineStr">
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="19" t="inlineStr">
         <is>
           <t>Bandbreite: In 50% der Fälle liegen die tatsächlichen Kosten innerhalb dieses Bereichs.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="20" t="inlineStr">
+    <row r="34" ht="26" customHeight="1">
+      <c r="A34" s="20" t="inlineStr">
         <is>
           <t>Bandbreite Gerichtskosten (±21%)</t>
         </is>
       </c>
-      <c r="B47" s="48">
+      <c r="B34" s="47">
         <f>B29*(1-0.21)</f>
         <v/>
       </c>
-      <c r="C47" s="48">
+      <c r="C34" s="47">
         <f>B29*(1+0.21)</f>
         <v/>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="20" t="inlineStr">
+    <row r="35" ht="26" customHeight="1">
+      <c r="A35" s="20" t="inlineStr">
         <is>
           <t>Bandbreite Parteientschädigung (±25.8%)</t>
         </is>
       </c>
-      <c r="B48" s="48">
+      <c r="B35" s="47">
         <f>B30*(1-0.258)</f>
         <v/>
       </c>
-      <c r="C48" s="48">
+      <c r="C35" s="47">
         <f>B30*(1+0.258)</f>
         <v/>
       </c>
     </row>
-    <row r="49"/>
-    <row r="50">
-      <c r="A50" s="13" t="inlineStr">
+    <row r="36" ht="6" customHeight="1"/>
+    <row r="37" ht="24" customHeight="1">
+      <c r="A37" s="13" t="inlineStr">
         <is>
           <t>Abweichung vom Tarif — Gerichtskosten</t>
         </is>
       </c>
-      <c r="B50" s="49">
+      <c r="B37" s="48">
         <f>(B29-B26)/B26</f>
         <v/>
       </c>
-      <c r="C50" s="15" t="inlineStr">
+      <c r="C37" s="15" t="inlineStr">
         <is>
           <t>positiv = über Tarif, negativ = unter Tarif</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="13" t="inlineStr">
+    <row r="38" ht="24" customHeight="1">
+      <c r="A38" s="13" t="inlineStr">
         <is>
           <t>Abweichung vom Tarif — Parteientschädigung</t>
         </is>
       </c>
-      <c r="B51" s="49">
+      <c r="B38" s="48">
         <f>(B30-B27)/B27</f>
         <v/>
       </c>
-      <c r="C51" s="15" t="inlineStr">
+      <c r="C38" s="15" t="inlineStr">
         <is>
           <t>positiv = über Tarif, negativ = unter Tarif</t>
         </is>
       </c>
     </row>
-    <row r="52"/>
-    <row r="53">
-      <c r="A53" s="23" t="inlineStr">
+    <row r="39" ht="10" customHeight="1"/>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="23" t="inlineStr">
         <is>
           <t>HAFTUNGSAUSSCHLUSS: Dieses Tool dient ausschliesslich zu Informations- und Bildungszwecken. Die Kostenschätzungen basieren auf statistischen Regressionsmodellen und empirischen Daten gemäss der Studie «From Tariff to Award». Die Ergebnisse sind Näherungswerte und können erheblich von den tatsächlich zugesprochenen Prozesskosten abweichen.
 Der Autor übernimmt keinerlei Haftung für die Richtigkeit, Vollständigkeit, Aktualität oder Zuverlässigkeit der mit diesem Tool generierten Schätzungen. Die Nutzung dieses Tools stellt keine Rechtsberatung dar. Es werden keinerlei Gewährleistungen abgegeben. Für fallspezifische Kosteneinschätzungen ist eine unabhängige fachkundige Beratung einzuholen.</t>
         </is>
       </c>
-      <c r="B53" s="50" t="n"/>
-      <c r="C53" s="51" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="52" t="n"/>
-      <c r="C54" s="53" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="52" t="n"/>
-      <c r="C55" s="53" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="52" t="n"/>
-      <c r="C56" s="53" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="54" t="n"/>
-      <c r="B57" s="55" t="n"/>
-      <c r="C57" s="56" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="19" t="inlineStr">
+      <c r="B40" s="49" t="n"/>
+      <c r="C40" s="50" t="n"/>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="51" t="n"/>
+      <c r="C41" s="52" t="n"/>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="51" t="n"/>
+      <c r="C42" s="52" t="n"/>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="51" t="n"/>
+      <c r="C43" s="52" t="n"/>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="53" t="n"/>
+      <c r="B44" s="54" t="n"/>
+      <c r="C44" s="55" t="n"/>
+    </row>
+    <row r="45" ht="16" customHeight="1">
+      <c r="A45" s="19" t="inlineStr">
         <is>
           <t>Grundlage: «From Tariff to Award» — Modell 6 (Year FE + Judge FE). Medianer abs. Prognosefehler: GK 21%, PE 25.8%.</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="25" t="inlineStr">
+    <row r="46" ht="16" customHeight="1">
+      <c r="A46" s="25" t="inlineStr">
         <is>
           <t>HILFSBERECHNUNGEN</t>
         </is>
       </c>
-      <c r="B59" s="26" t="n"/>
-      <c r="C59" s="26" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="27" t="inlineStr">
+      <c r="B46" s="26" t="n"/>
+      <c r="C46" s="26" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="27" t="inlineStr">
         <is>
           <t>ln(GK / Grundtarif)</t>
         </is>
       </c>
-      <c r="B60" s="57">
+      <c r="B47" s="56">
         <f>Koeffizienten!B3+LN(B26)*Koeffizienten!B4+IF(B7="Aargau",1,0)*Koeffizienten!B5+IF(B7="Aargau",1,0)*LN(B26)*Koeffizienten!B6+INDEX(Koeffizienten!B$31:B$39,MATCH(B9,Koeffizienten!A$31:A$39,0))+IF(B10="Ja",1,0)*Koeffizienten!B9+IF(B11="Ja",1,0)*Koeffizienten!B10+LN(MAX(1,B12))*Koeffizienten!B7+LN(MAX(1,B13))*Koeffizienten!B8+IF(B15="Ja",1,0)*Koeffizienten!B19+IF(B16="Ja",1,0)*Koeffizienten!B20+IF(B17="Ja",1,0)*Koeffizienten!B21+IF(B18="Ja",1,0)*Koeffizienten!B22+IF(B19="Ja",1,0)*Koeffizienten!B23+IF(B20="Ja",1,0)*Koeffizienten!B24+IF(B21="Ja",1,0)*Koeffizienten!B25</f>
         <v/>
       </c>
-      <c r="C60" s="26" t="n"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="27" t="inlineStr">
+      <c r="C47" s="26" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="27" t="inlineStr">
         <is>
           <t>ln(PE / Grundtarif)</t>
         </is>
       </c>
-      <c r="B61" s="57">
+      <c r="B48" s="56">
         <f>Koeffizienten!C3+LN(B27)*Koeffizienten!C4+IF(B7="Aargau",1,0)*Koeffizienten!C5+IF(B7="Aargau",1,0)*LN(B27)*Koeffizienten!C6+INDEX(Koeffizienten!C$31:C$39,MATCH(B9,Koeffizienten!A$31:A$39,0))+IF(B10="Ja",1,0)*Koeffizienten!C9+IF(B11="Ja",1,0)*Koeffizienten!C10+LN(MAX(1,B12))*Koeffizienten!C7+LN(MAX(1,B13))*Koeffizienten!C8+IF(B15="Ja",1,0)*Koeffizienten!C19+IF(B16="Ja",1,0)*Koeffizienten!C20+IF(B17="Ja",1,0)*Koeffizienten!C21+IF(B18="Ja",1,0)*Koeffizienten!C22+IF(B19="Ja",1,0)*Koeffizienten!C23+IF(B20="Ja",1,0)*Koeffizienten!C24+IF(B21="Ja",1,0)*Koeffizienten!C25+B23*Koeffizienten!C26</f>
         <v/>
       </c>
-      <c r="C61" s="26" t="n"/>
+      <c r="C48" s="26" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="8">
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="A33:C33"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A45:C45"/>
-    <mergeCell ref="A1:C1"/>
     <mergeCell ref="A40:C44"/>
     <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A8:C11"/>
-    <mergeCell ref="A2:C5"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
@@ -1480,7 +1461,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="003574A7"/>
@@ -1565,7 +1546,7 @@
       <c r="C3" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="D3" s="58" t="n">
+      <c r="D3" s="57" t="n">
         <v>0.25</v>
       </c>
       <c r="F3" s="31" t="n">
@@ -1577,7 +1558,7 @@
       <c r="H3" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="I3" s="58" t="n">
+      <c r="I3" s="57" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -1591,7 +1572,7 @@
       <c r="C4" s="33" t="n">
         <v>250</v>
       </c>
-      <c r="D4" s="59" t="n">
+      <c r="D4" s="58" t="n">
         <v>0.2</v>
       </c>
       <c r="F4" s="33" t="n">
@@ -1603,7 +1584,7 @@
       <c r="H4" s="33" t="n">
         <v>1250</v>
       </c>
-      <c r="I4" s="59" t="n">
+      <c r="I4" s="58" t="n">
         <v>0.23</v>
       </c>
     </row>
@@ -1617,7 +1598,7 @@
       <c r="C5" s="31" t="n">
         <v>1050</v>
       </c>
-      <c r="D5" s="58" t="n">
+      <c r="D5" s="57" t="n">
         <v>0.14</v>
       </c>
       <c r="F5" s="31" t="n">
@@ -1629,7 +1610,7 @@
       <c r="H5" s="31" t="n">
         <v>2400</v>
       </c>
-      <c r="I5" s="58" t="n">
+      <c r="I5" s="57" t="n">
         <v>0.15</v>
       </c>
     </row>
@@ -1643,7 +1624,7 @@
       <c r="C6" s="33" t="n">
         <v>3150</v>
       </c>
-      <c r="D6" s="59" t="n">
+      <c r="D6" s="58" t="n">
         <v>0.08</v>
       </c>
       <c r="F6" s="33" t="n">
@@ -1655,7 +1636,7 @@
       <c r="H6" s="33" t="n">
         <v>3900</v>
       </c>
-      <c r="I6" s="59" t="n">
+      <c r="I6" s="58" t="n">
         <v>0.11</v>
       </c>
     </row>
@@ -1669,7 +1650,7 @@
       <c r="C7" s="31" t="n">
         <v>7950</v>
       </c>
-      <c r="D7" s="58" t="n">
+      <c r="D7" s="57" t="n">
         <v>0.04</v>
       </c>
       <c r="F7" s="31" t="n">
@@ -1681,7 +1662,7 @@
       <c r="H7" s="31" t="n">
         <v>6100</v>
       </c>
-      <c r="I7" s="58" t="n">
+      <c r="I7" s="57" t="n">
         <v>0.09</v>
       </c>
     </row>
@@ -1695,7 +1676,7 @@
       <c r="C8" s="33" t="n">
         <v>16750</v>
       </c>
-      <c r="D8" s="59" t="n">
+      <c r="D8" s="58" t="n">
         <v>0.02</v>
       </c>
       <c r="F8" s="33" t="n">
@@ -1707,7 +1688,7 @@
       <c r="H8" s="33" t="n">
         <v>9700</v>
       </c>
-      <c r="I8" s="59" t="n">
+      <c r="I8" s="58" t="n">
         <v>0.06</v>
       </c>
     </row>
@@ -1721,7 +1702,7 @@
       <c r="C9" s="31" t="n">
         <v>30750</v>
       </c>
-      <c r="D9" s="58" t="n">
+      <c r="D9" s="57" t="n">
         <v>0.01</v>
       </c>
       <c r="F9" s="31" t="n">
@@ -1733,7 +1714,7 @@
       <c r="H9" s="31" t="n">
         <v>14500</v>
       </c>
-      <c r="I9" s="58" t="n">
+      <c r="I9" s="57" t="n">
         <v>0.035</v>
       </c>
     </row>
@@ -1747,7 +1728,7 @@
       <c r="C10" s="33" t="n">
         <v>120750</v>
       </c>
-      <c r="D10" s="59" t="n">
+      <c r="D10" s="58" t="n">
         <v>0.005</v>
       </c>
       <c r="F10" s="33" t="n">
@@ -1759,7 +1740,7 @@
       <c r="H10" s="33" t="n">
         <v>19400</v>
       </c>
-      <c r="I10" s="59" t="n">
+      <c r="I10" s="58" t="n">
         <v>0.02</v>
       </c>
     </row>
@@ -1773,7 +1754,7 @@
       <c r="H11" s="31" t="n">
         <v>25400</v>
       </c>
-      <c r="I11" s="58" t="n">
+      <c r="I11" s="57" t="n">
         <v>0.015</v>
       </c>
     </row>
@@ -1787,7 +1768,7 @@
       <c r="H12" s="33" t="n">
         <v>31400</v>
       </c>
-      <c r="I12" s="59" t="n">
+      <c r="I12" s="58" t="n">
         <v>0.01</v>
       </c>
     </row>
@@ -1801,7 +1782,7 @@
       <c r="H13" s="31" t="n">
         <v>61400</v>
       </c>
-      <c r="I13" s="58" t="n">
+      <c r="I13" s="57" t="n">
         <v>0.0075</v>
       </c>
     </row>
@@ -1815,7 +1796,7 @@
       <c r="H14" s="33" t="n">
         <v>106400</v>
       </c>
-      <c r="I14" s="59" t="n">
+      <c r="I14" s="58" t="n">
         <v>0.005</v>
       </c>
     </row>
@@ -1883,7 +1864,7 @@
       <c r="C19" s="31" t="n">
         <v>900</v>
       </c>
-      <c r="D19" s="58" t="n">
+      <c r="D19" s="57" t="n">
         <v>0.11</v>
       </c>
       <c r="F19" s="31" t="n">
@@ -1895,7 +1876,7 @@
       <c r="H19" s="31" t="n">
         <v>1110</v>
       </c>
-      <c r="I19" s="58" t="n">
+      <c r="I19" s="57" t="n">
         <v>0.22</v>
       </c>
     </row>
@@ -1909,7 +1890,7 @@
       <c r="C20" s="33" t="n">
         <v>1160</v>
       </c>
-      <c r="D20" s="59" t="n">
+      <c r="D20" s="58" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="F20" s="33" t="n">
@@ -1921,7 +1902,7 @@
       <c r="H20" s="33" t="n">
         <v>1230</v>
       </c>
-      <c r="I20" s="59" t="n">
+      <c r="I20" s="58" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -1935,7 +1916,7 @@
       <c r="C21" s="31" t="n">
         <v>1290</v>
       </c>
-      <c r="D21" s="58" t="n">
+      <c r="D21" s="57" t="n">
         <v>0.06</v>
       </c>
       <c r="F21" s="31" t="n">
@@ -1947,7 +1928,7 @@
       <c r="H21" s="31" t="n">
         <v>1850</v>
       </c>
-      <c r="I21" s="58" t="n">
+      <c r="I21" s="57" t="n">
         <v>0.15</v>
       </c>
     </row>
@@ -1961,7 +1942,7 @@
       <c r="C22" s="33" t="n">
         <v>770</v>
       </c>
-      <c r="D22" s="59" t="n">
+      <c r="D22" s="58" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="F22" s="33" t="n">
@@ -1973,7 +1954,7 @@
       <c r="H22" s="33" t="n">
         <v>2590</v>
       </c>
-      <c r="I22" s="59" t="n">
+      <c r="I22" s="58" t="n">
         <v>0.12</v>
       </c>
     </row>
@@ -1987,7 +1968,7 @@
       <c r="C23" s="31" t="n">
         <v>4270</v>
       </c>
-      <c r="D23" s="58" t="n">
+      <c r="D23" s="57" t="n">
         <v>0.035</v>
       </c>
       <c r="F23" s="31" t="n">
@@ -1999,7 +1980,7 @@
       <c r="H23" s="31" t="n">
         <v>4070</v>
       </c>
-      <c r="I23" s="58" t="n">
+      <c r="I23" s="57" t="n">
         <v>0.09</v>
       </c>
     </row>
@@ -2013,7 +1994,7 @@
       <c r="C24" s="33" t="n">
         <v>6870</v>
       </c>
-      <c r="D24" s="59" t="n">
+      <c r="D24" s="58" t="n">
         <v>0.022</v>
       </c>
       <c r="F24" s="33" t="n">
@@ -2025,7 +2006,7 @@
       <c r="H24" s="33" t="n">
         <v>6530</v>
       </c>
-      <c r="I24" s="59" t="n">
+      <c r="I24" s="58" t="n">
         <v>0.064</v>
       </c>
     </row>
@@ -2039,7 +2020,7 @@
       <c r="C25" s="31" t="n">
         <v>9670</v>
       </c>
-      <c r="D25" s="58" t="n">
+      <c r="D25" s="57" t="n">
         <v>0.015</v>
       </c>
       <c r="F25" s="31" t="n">
@@ -2051,7 +2032,7 @@
       <c r="H25" s="31" t="n">
         <v>10230</v>
       </c>
-      <c r="I25" s="58" t="n">
+      <c r="I25" s="57" t="n">
         <v>0.044</v>
       </c>
     </row>
@@ -2065,7 +2046,7 @@
       <c r="C26" s="33" t="n">
         <v>13670</v>
       </c>
-      <c r="D26" s="59" t="n">
+      <c r="D26" s="58" t="n">
         <v>0.01</v>
       </c>
       <c r="F26" s="33" t="n">
@@ -2077,7 +2058,7 @@
       <c r="H26" s="33" t="n">
         <v>14300</v>
       </c>
-      <c r="I26" s="59" t="n">
+      <c r="I26" s="58" t="n">
         <v>0.033</v>
       </c>
     </row>
@@ -2091,7 +2072,7 @@
       <c r="C27" s="31" t="n">
         <v>21670</v>
       </c>
-      <c r="D27" s="58" t="n">
+      <c r="D27" s="57" t="n">
         <v>0.005</v>
       </c>
       <c r="F27" s="31" t="n">
@@ -2103,7 +2084,7 @@
       <c r="H27" s="31" t="n">
         <v>20240</v>
       </c>
-      <c r="I27" s="58" t="n">
+      <c r="I27" s="57" t="n">
         <v>0.025</v>
       </c>
     </row>
@@ -2117,7 +2098,7 @@
       <c r="C28" s="33" t="n">
         <v>28270</v>
       </c>
-      <c r="D28" s="59" t="n">
+      <c r="D28" s="58" t="n">
         <v>0.003</v>
       </c>
       <c r="F28" s="33" t="n">
@@ -2129,7 +2110,7 @@
       <c r="H28" s="33" t="n">
         <v>29040</v>
       </c>
-      <c r="I28" s="59" t="n">
+      <c r="I28" s="58" t="n">
         <v>0.019</v>
       </c>
     </row>
@@ -2143,7 +2124,7 @@
       <c r="H29" s="31" t="n">
         <v>44440</v>
       </c>
-      <c r="I29" s="58" t="n">
+      <c r="I29" s="57" t="n">
         <v>0.014</v>
       </c>
     </row>
@@ -2157,7 +2138,7 @@
       <c r="H30" s="33" t="n">
         <v>69080</v>
       </c>
-      <c r="I30" s="59" t="n">
+      <c r="I30" s="58" t="n">
         <v>0.01</v>
       </c>
     </row>
@@ -2188,7 +2169,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00548235"/>
@@ -2233,10 +2214,10 @@
           <t>Intercept</t>
         </is>
       </c>
-      <c r="B3" s="60" t="n">
+      <c r="B3" s="59" t="n">
         <v>0.927</v>
       </c>
-      <c r="C3" s="60" t="n">
+      <c r="C3" s="59" t="n">
         <v>1.888</v>
       </c>
     </row>
@@ -2246,10 +2227,10 @@
           <t>ln(Baseline)</t>
         </is>
       </c>
-      <c r="B4" s="61" t="n">
+      <c r="B4" s="60" t="n">
         <v>-0.111</v>
       </c>
-      <c r="C4" s="61" t="n">
+      <c r="C4" s="60" t="n">
         <v>-0.17</v>
       </c>
     </row>
@@ -2259,10 +2240,10 @@
           <t>D_AG</t>
         </is>
       </c>
-      <c r="B5" s="60" t="n">
+      <c r="B5" s="59" t="n">
         <v>-0.518</v>
       </c>
-      <c r="C5" s="60" t="n">
+      <c r="C5" s="59" t="n">
         <v>-3.414</v>
       </c>
     </row>
@@ -2272,10 +2253,10 @@
           <t>D_AG x ln(Baseline)</t>
         </is>
       </c>
-      <c r="B6" s="61" t="n">
+      <c r="B6" s="60" t="n">
         <v>0.057</v>
       </c>
-      <c r="C6" s="61" t="n">
+      <c r="C6" s="60" t="n">
         <v>0.463</v>
       </c>
     </row>
@@ -2285,10 +2266,10 @@
           <t>ln(Kläger)</t>
         </is>
       </c>
-      <c r="B7" s="60" t="n">
+      <c r="B7" s="59" t="n">
         <v>0.052</v>
       </c>
-      <c r="C7" s="60" t="n">
+      <c r="C7" s="59" t="n">
         <v>-0.13</v>
       </c>
     </row>
@@ -2298,10 +2279,10 @@
           <t>ln(Beklagte)</t>
         </is>
       </c>
-      <c r="B8" s="61" t="n">
+      <c r="B8" s="60" t="n">
         <v>0.092</v>
       </c>
-      <c r="C8" s="61" t="n">
+      <c r="C8" s="60" t="n">
         <v>0.176</v>
       </c>
     </row>
@@ -2311,10 +2292,10 @@
           <t>Domizil Kläger</t>
         </is>
       </c>
-      <c r="B9" s="60" t="n">
+      <c r="B9" s="59" t="n">
         <v>-0.08599999999999999</v>
       </c>
-      <c r="C9" s="60" t="n">
+      <c r="C9" s="59" t="n">
         <v>-0.129</v>
       </c>
     </row>
@@ -2324,10 +2305,10 @@
           <t>Domizil Beklagter</t>
         </is>
       </c>
-      <c r="B10" s="61" t="n">
+      <c r="B10" s="60" t="n">
         <v>-0.079</v>
       </c>
-      <c r="C10" s="61" t="n">
+      <c r="C10" s="60" t="n">
         <v>-0.022</v>
       </c>
     </row>
@@ -2337,10 +2318,10 @@
           <t>D_Bau</t>
         </is>
       </c>
-      <c r="B11" s="60" t="n">
+      <c r="B11" s="59" t="n">
         <v>0.037</v>
       </c>
-      <c r="C11" s="60" t="n">
+      <c r="C11" s="59" t="n">
         <v>-0.208</v>
       </c>
     </row>
@@ -2350,10 +2331,10 @@
           <t>D_Handel</t>
         </is>
       </c>
-      <c r="B12" s="61" t="n">
+      <c r="B12" s="60" t="n">
         <v>0.007</v>
       </c>
-      <c r="C12" s="61" t="n">
+      <c r="C12" s="60" t="n">
         <v>0.004</v>
       </c>
     </row>
@@ -2363,10 +2344,10 @@
           <t>D_Finanz/Versicherung</t>
         </is>
       </c>
-      <c r="B13" s="60" t="n">
+      <c r="B13" s="59" t="n">
         <v>0.068</v>
       </c>
-      <c r="C13" s="60" t="n">
+      <c r="C13" s="59" t="n">
         <v>-0.12</v>
       </c>
     </row>
@@ -2376,10 +2357,10 @@
           <t>D_Organhaftung</t>
         </is>
       </c>
-      <c r="B14" s="61" t="n">
+      <c r="B14" s="60" t="n">
         <v>-0.006</v>
       </c>
-      <c r="C14" s="61" t="n">
+      <c r="C14" s="60" t="n">
         <v>-0.064</v>
       </c>
     </row>
@@ -2389,10 +2370,10 @@
           <t>D_UWG/URG</t>
         </is>
       </c>
-      <c r="B15" s="60" t="n">
+      <c r="B15" s="59" t="n">
         <v>0.592</v>
       </c>
-      <c r="C15" s="60" t="n">
+      <c r="C15" s="59" t="n">
         <v>1.058</v>
       </c>
     </row>
@@ -2402,10 +2383,10 @@
           <t>D_Immaterialgüterrecht</t>
         </is>
       </c>
-      <c r="B16" s="61" t="n">
+      <c r="B16" s="60" t="n">
         <v>0.06900000000000001</v>
       </c>
-      <c r="C16" s="61" t="n">
+      <c r="C16" s="60" t="n">
         <v>-0.079</v>
       </c>
     </row>
@@ -2415,10 +2396,10 @@
           <t>D_Gesellschaftsrecht</t>
         </is>
       </c>
-      <c r="B17" s="60" t="n">
+      <c r="B17" s="59" t="n">
         <v>-0.227</v>
       </c>
-      <c r="C17" s="60" t="n">
+      <c r="C17" s="59" t="n">
         <v>-0.045</v>
       </c>
     </row>
@@ -2428,10 +2409,10 @@
           <t>D_Übrige</t>
         </is>
       </c>
-      <c r="B18" s="61" t="n">
+      <c r="B18" s="60" t="n">
         <v>0.029</v>
       </c>
-      <c r="C18" s="61" t="n">
+      <c r="C18" s="60" t="n">
         <v>-0.159</v>
       </c>
     </row>
@@ -2441,10 +2422,10 @@
           <t>Klagantwort</t>
         </is>
       </c>
-      <c r="B19" s="60" t="n">
+      <c r="B19" s="59" t="n">
         <v>-0.08799999999999999</v>
       </c>
-      <c r="C19" s="60" t="n">
+      <c r="C19" s="59" t="n">
         <v>-0.004</v>
       </c>
     </row>
@@ -2454,10 +2435,10 @@
           <t>Zweiter Schriftenwechsel</t>
         </is>
       </c>
-      <c r="B20" s="61" t="n">
+      <c r="B20" s="60" t="n">
         <v>0.504</v>
       </c>
-      <c r="C20" s="61" t="n">
+      <c r="C20" s="60" t="n">
         <v>0.319</v>
       </c>
     </row>
@@ -2467,10 +2448,10 @@
           <t>Widerklage</t>
         </is>
       </c>
-      <c r="B21" s="60" t="n">
+      <c r="B21" s="59" t="n">
         <v>-0.159</v>
       </c>
-      <c r="C21" s="60" t="n">
+      <c r="C21" s="59" t="n">
         <v>-0.173</v>
       </c>
     </row>
@@ -2480,10 +2461,10 @@
           <t>Widerklage 2. SW</t>
         </is>
       </c>
-      <c r="B22" s="61" t="n">
+      <c r="B22" s="60" t="n">
         <v>0.395</v>
       </c>
-      <c r="C22" s="61" t="n">
+      <c r="C22" s="60" t="n">
         <v>0.192</v>
       </c>
     </row>
@@ -2493,10 +2474,10 @@
           <t>Zusätzliche Eingaben</t>
         </is>
       </c>
-      <c r="B23" s="60" t="n">
+      <c r="B23" s="59" t="n">
         <v>0.051</v>
       </c>
-      <c r="C23" s="60" t="n">
+      <c r="C23" s="59" t="n">
         <v>0.147</v>
       </c>
     </row>
@@ -2506,10 +2487,10 @@
           <t>Vergleichsverhandlung</t>
         </is>
       </c>
-      <c r="B24" s="61" t="n">
+      <c r="B24" s="60" t="n">
         <v>0.15</v>
       </c>
-      <c r="C24" s="61" t="n">
+      <c r="C24" s="60" t="n">
         <v>0.023</v>
       </c>
     </row>
@@ -2519,10 +2500,10 @@
           <t>Gutachten</t>
         </is>
       </c>
-      <c r="B25" s="60" t="n">
+      <c r="B25" s="59" t="n">
         <v>0.123</v>
       </c>
-      <c r="C25" s="60" t="n">
+      <c r="C25" s="59" t="n">
         <v>-0.319</v>
       </c>
     </row>
@@ -2532,10 +2513,10 @@
           <t>Unterliegensquote Kläger</t>
         </is>
       </c>
-      <c r="B26" s="61" t="n">
+      <c r="B26" s="60" t="n">
         <v>0</v>
       </c>
-      <c r="C26" s="61" t="n">
+      <c r="C26" s="60" t="n">
         <v>0.122</v>
       </c>
     </row>
@@ -2570,10 +2551,10 @@
           <t>Forderung Dienstleistungen</t>
         </is>
       </c>
-      <c r="B31" s="60" t="n">
+      <c r="B31" s="59" t="n">
         <v>0</v>
       </c>
-      <c r="C31" s="60" t="n">
+      <c r="C31" s="59" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2583,10 +2564,10 @@
           <t>Forderung Bau</t>
         </is>
       </c>
-      <c r="B32" s="61" t="n">
+      <c r="B32" s="60" t="n">
         <v>0.037</v>
       </c>
-      <c r="C32" s="61" t="n">
+      <c r="C32" s="60" t="n">
         <v>-0.208</v>
       </c>
     </row>
@@ -2596,10 +2577,10 @@
           <t>Forderung Handel</t>
         </is>
       </c>
-      <c r="B33" s="60" t="n">
+      <c r="B33" s="59" t="n">
         <v>0.007</v>
       </c>
-      <c r="C33" s="60" t="n">
+      <c r="C33" s="59" t="n">
         <v>0.004</v>
       </c>
     </row>
@@ -2609,10 +2590,10 @@
           <t>Forderung Finanz/Versicherung</t>
         </is>
       </c>
-      <c r="B34" s="61" t="n">
+      <c r="B34" s="60" t="n">
         <v>0.068</v>
       </c>
-      <c r="C34" s="61" t="n">
+      <c r="C34" s="60" t="n">
         <v>-0.12</v>
       </c>
     </row>
@@ -2622,10 +2603,10 @@
           <t>Haftung Gesellschaftsorgane</t>
         </is>
       </c>
-      <c r="B35" s="60" t="n">
+      <c r="B35" s="59" t="n">
         <v>-0.006</v>
       </c>
-      <c r="C35" s="60" t="n">
+      <c r="C35" s="59" t="n">
         <v>-0.064</v>
       </c>
     </row>
@@ -2635,10 +2616,10 @@
           <t>UWG/URG</t>
         </is>
       </c>
-      <c r="B36" s="61" t="n">
+      <c r="B36" s="60" t="n">
         <v>0.592</v>
       </c>
-      <c r="C36" s="61" t="n">
+      <c r="C36" s="60" t="n">
         <v>1.058</v>
       </c>
     </row>
@@ -2648,10 +2629,10 @@
           <t>Immaterialgüterrecht</t>
         </is>
       </c>
-      <c r="B37" s="60" t="n">
+      <c r="B37" s="59" t="n">
         <v>0.06900000000000001</v>
       </c>
-      <c r="C37" s="60" t="n">
+      <c r="C37" s="59" t="n">
         <v>-0.079</v>
       </c>
     </row>
@@ -2661,10 +2642,10 @@
           <t>Gesellschaftsrecht</t>
         </is>
       </c>
-      <c r="B38" s="61" t="n">
+      <c r="B38" s="60" t="n">
         <v>-0.227</v>
       </c>
-      <c r="C38" s="61" t="n">
+      <c r="C38" s="60" t="n">
         <v>-0.045</v>
       </c>
     </row>
@@ -2674,10 +2655,10 @@
           <t>Übrige</t>
         </is>
       </c>
-      <c r="B39" s="60" t="n">
+      <c r="B39" s="59" t="n">
         <v>0.029</v>
       </c>
-      <c r="C39" s="60" t="n">
+      <c r="C39" s="59" t="n">
         <v>-0.159</v>
       </c>
     </row>

</xml_diff>